<commit_message>
feat: enhance extraction prompt, add EPD carbon calculations (B2), and optimize visualization to use JSON
</commit_message>
<xml_diff>
--- a/output/passport_filled.xlsx
+++ b/output/passport_filled.xlsx
@@ -1216,12 +1216,12 @@
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>Earth</t>
+          <t>Soil</t>
         </is>
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>Earth</t>
+          <t>Soil</t>
         </is>
       </c>
       <c r="J8" s="8" t="inlineStr">
@@ -1310,12 +1310,12 @@
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
+          <t>Fine sand</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
           <t>Sand</t>
-        </is>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Fine sand</t>
         </is>
       </c>
       <c r="J9" s="8" t="inlineStr">
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="K10" s="17" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="L10" s="8" t="n"/>
       <c r="M10" s="8" t="n"/>
@@ -1577,7 +1577,7 @@
       <c r="F12" s="8" t="n"/>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Civil &amp; Sitework</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
-          <t>Cement, Coarse sand, Graded stone aggregate</t>
+          <t>Cement, Coarse sand, Stone aggregate</t>
         </is>
       </c>
       <c r="J12" s="8" t="inlineStr">
@@ -1596,7 +1596,7 @@
         </is>
       </c>
       <c r="K12" s="17" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="L12" s="8" t="n"/>
       <c r="M12" s="8" t="inlineStr">
@@ -1623,8 +1623,12 @@
       <c r="V12" s="8" t="n"/>
       <c r="W12" s="8" t="n"/>
       <c r="X12" s="8" t="n"/>
-      <c r="Y12" s="8" t="n"/>
-      <c r="Z12" s="8" t="n"/>
+      <c r="Y12" s="17" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="Z12" s="17" t="n">
+        <v>0.149</v>
+      </c>
       <c r="AA12" s="8" t="n"/>
       <c r="AB12" s="8" t="inlineStr">
         <is>
@@ -1652,7 +1656,11 @@
       <c r="AU12" s="8" t="n"/>
       <c r="AV12" s="8" t="n"/>
       <c r="AW12" s="8" t="n"/>
-      <c r="AX12" s="8" t="n"/>
+      <c r="AX12" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="n"/>
@@ -1671,7 +1679,7 @@
       <c r="F13" s="8" t="n"/>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Civil &amp; Sitework</t>
         </is>
       </c>
       <c r="H13" s="8" t="inlineStr">
@@ -1681,7 +1689,7 @@
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>Cement, Fine sand, Graded stone aggregate</t>
+          <t>Cement, Fine sand, Stone aggregate</t>
         </is>
       </c>
       <c r="J13" s="8" t="inlineStr">
@@ -1690,7 +1698,7 @@
         </is>
       </c>
       <c r="K13" s="17" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="L13" s="8" t="n"/>
       <c r="M13" s="8" t="inlineStr">
@@ -1717,8 +1725,12 @@
       <c r="V13" s="8" t="n"/>
       <c r="W13" s="8" t="n"/>
       <c r="X13" s="8" t="n"/>
-      <c r="Y13" s="8" t="n"/>
-      <c r="Z13" s="8" t="n"/>
+      <c r="Y13" s="17" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="Z13" s="17" t="n">
+        <v>0.149</v>
+      </c>
       <c r="AA13" s="8" t="n"/>
       <c r="AB13" s="8" t="inlineStr">
         <is>
@@ -1746,7 +1758,11 @@
       <c r="AU13" s="8" t="n"/>
       <c r="AV13" s="8" t="n"/>
       <c r="AW13" s="8" t="n"/>
-      <c r="AX13" s="8" t="n"/>
+      <c r="AX13" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n"/>
@@ -1765,7 +1781,7 @@
       <c r="F14" s="8" t="n"/>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Civil &amp; Sitework</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
@@ -1775,7 +1791,7 @@
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>Cement, Coarse sand, Graded stone aggregate</t>
+          <t>Cement, Coarse sand, Stone aggregate</t>
         </is>
       </c>
       <c r="J14" s="8" t="inlineStr">
@@ -1784,7 +1800,7 @@
         </is>
       </c>
       <c r="K14" s="17" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="L14" s="8" t="n"/>
       <c r="M14" s="8" t="inlineStr">
@@ -1811,8 +1827,12 @@
       <c r="V14" s="8" t="n"/>
       <c r="W14" s="8" t="n"/>
       <c r="X14" s="8" t="n"/>
-      <c r="Y14" s="8" t="n"/>
-      <c r="Z14" s="8" t="n"/>
+      <c r="Y14" s="17" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="Z14" s="17" t="n">
+        <v>0.149</v>
+      </c>
       <c r="AA14" s="8" t="n"/>
       <c r="AB14" s="8" t="inlineStr">
         <is>
@@ -1840,7 +1860,11 @@
       <c r="AU14" s="8" t="n"/>
       <c r="AV14" s="8" t="n"/>
       <c r="AW14" s="8" t="n"/>
-      <c r="AX14" s="8" t="n"/>
+      <c r="AX14" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n"/>
@@ -1869,7 +1893,7 @@
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>Cement, Coarse sand, Graded stone aggregate</t>
+          <t>Cement, Coarse sand, Stone aggregate</t>
         </is>
       </c>
       <c r="J15" s="8" t="inlineStr">
@@ -1905,8 +1929,12 @@
       <c r="V15" s="8" t="n"/>
       <c r="W15" s="8" t="n"/>
       <c r="X15" s="8" t="n"/>
-      <c r="Y15" s="8" t="n"/>
-      <c r="Z15" s="8" t="n"/>
+      <c r="Y15" s="17" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="Z15" s="17" t="n">
+        <v>0.149</v>
+      </c>
       <c r="AA15" s="8" t="n"/>
       <c r="AB15" s="8" t="inlineStr">
         <is>
@@ -1936,7 +1964,11 @@
       <c r="AU15" s="8" t="n"/>
       <c r="AV15" s="8" t="n"/>
       <c r="AW15" s="8" t="n"/>
-      <c r="AX15" s="8" t="n"/>
+      <c r="AX15" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n"/>
@@ -1965,7 +1997,7 @@
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>Petroleum bitumen, Kerosene oil</t>
+          <t>Bitumen, Kerosene oil</t>
         </is>
       </c>
       <c r="J16" s="8" t="inlineStr">
@@ -2055,7 +2087,7 @@
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>Cement, Coarse sand, Graded stone aggregate</t>
+          <t>Cement, Coarse sand, Stone aggregate</t>
         </is>
       </c>
       <c r="J17" s="8" t="inlineStr">
@@ -2064,7 +2096,7 @@
         </is>
       </c>
       <c r="K17" s="17" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="L17" s="8" t="n"/>
       <c r="M17" s="8" t="inlineStr">
@@ -2091,8 +2123,12 @@
       <c r="V17" s="8" t="n"/>
       <c r="W17" s="8" t="n"/>
       <c r="X17" s="8" t="n"/>
-      <c r="Y17" s="8" t="n"/>
-      <c r="Z17" s="8" t="n"/>
+      <c r="Y17" s="17" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="Z17" s="17" t="n">
+        <v>0.149</v>
+      </c>
       <c r="AA17" s="8" t="n"/>
       <c r="AB17" s="8" t="inlineStr">
         <is>
@@ -2120,7 +2156,11 @@
       <c r="AU17" s="8" t="n"/>
       <c r="AV17" s="8" t="n"/>
       <c r="AW17" s="8" t="n"/>
-      <c r="AX17" s="8" t="n"/>
+      <c r="AX17" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n"/>
@@ -2149,7 +2189,7 @@
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>Cement, Coarse sand, Graded stone aggregate</t>
+          <t>Cement, Coarse sand, Stone aggregate</t>
         </is>
       </c>
       <c r="J18" s="8" t="inlineStr">
@@ -2158,7 +2198,7 @@
         </is>
       </c>
       <c r="K18" s="17" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="L18" s="8" t="n"/>
       <c r="M18" s="8" t="inlineStr">
@@ -2185,8 +2225,12 @@
       <c r="V18" s="8" t="n"/>
       <c r="W18" s="8" t="n"/>
       <c r="X18" s="8" t="n"/>
-      <c r="Y18" s="8" t="n"/>
-      <c r="Z18" s="8" t="n"/>
+      <c r="Y18" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Z18" s="17" t="n">
+        <v>0.149</v>
+      </c>
       <c r="AA18" s="8" t="n"/>
       <c r="AB18" s="8" t="inlineStr">
         <is>
@@ -2214,7 +2258,11 @@
       <c r="AU18" s="8" t="n"/>
       <c r="AV18" s="8" t="n"/>
       <c r="AW18" s="8" t="n"/>
-      <c r="AX18" s="8" t="n"/>
+      <c r="AX18" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="n"/>
@@ -2243,7 +2291,7 @@
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>Cement, Coarse sand, Graded stone aggregate</t>
+          <t>Cement, Coarse sand, Stone aggregate</t>
         </is>
       </c>
       <c r="J19" s="8" t="inlineStr">
@@ -2252,7 +2300,7 @@
         </is>
       </c>
       <c r="K19" s="17" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="L19" s="8" t="n"/>
       <c r="M19" s="8" t="inlineStr">
@@ -2279,8 +2327,12 @@
       <c r="V19" s="8" t="n"/>
       <c r="W19" s="8" t="n"/>
       <c r="X19" s="8" t="n"/>
-      <c r="Y19" s="8" t="n"/>
-      <c r="Z19" s="8" t="n"/>
+      <c r="Y19" s="17" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="Z19" s="17" t="n">
+        <v>0.149</v>
+      </c>
       <c r="AA19" s="8" t="n"/>
       <c r="AB19" s="8" t="inlineStr">
         <is>
@@ -2308,7 +2360,11 @@
       <c r="AU19" s="8" t="n"/>
       <c r="AV19" s="8" t="n"/>
       <c r="AW19" s="8" t="n"/>
-      <c r="AX19" s="8" t="n"/>
+      <c r="AX19" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n"/>
@@ -2337,7 +2393,7 @@
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>Cement, Coarse sand, Graded stone aggregate</t>
+          <t>Cement, Coarse sand, Stone aggregate</t>
         </is>
       </c>
       <c r="J20" s="8" t="inlineStr">
@@ -2346,7 +2402,7 @@
         </is>
       </c>
       <c r="K20" s="17" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="L20" s="8" t="n"/>
       <c r="M20" s="8" t="inlineStr">
@@ -2373,8 +2429,12 @@
       <c r="V20" s="8" t="n"/>
       <c r="W20" s="8" t="n"/>
       <c r="X20" s="8" t="n"/>
-      <c r="Y20" s="8" t="n"/>
-      <c r="Z20" s="8" t="n"/>
+      <c r="Y20" s="17" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Z20" s="17" t="n">
+        <v>0.149</v>
+      </c>
       <c r="AA20" s="8" t="n"/>
       <c r="AB20" s="8" t="inlineStr">
         <is>
@@ -2402,7 +2462,11 @@
       <c r="AU20" s="8" t="n"/>
       <c r="AV20" s="8" t="n"/>
       <c r="AW20" s="8" t="n"/>
-      <c r="AX20" s="8" t="n"/>
+      <c r="AX20" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="n"/>
@@ -2431,7 +2495,7 @@
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>Cement, Coarse sand, Graded stone aggregate</t>
+          <t>Cement, Coarse sand, Stone aggregate</t>
         </is>
       </c>
       <c r="J21" s="8" t="inlineStr">
@@ -2440,7 +2504,7 @@
         </is>
       </c>
       <c r="K21" s="17" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="L21" s="8" t="n"/>
       <c r="M21" s="8" t="inlineStr">
@@ -2467,8 +2531,12 @@
       <c r="V21" s="8" t="n"/>
       <c r="W21" s="8" t="n"/>
       <c r="X21" s="8" t="n"/>
-      <c r="Y21" s="8" t="n"/>
-      <c r="Z21" s="8" t="n"/>
+      <c r="Y21" s="17" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="Z21" s="17" t="n">
+        <v>0.149</v>
+      </c>
       <c r="AA21" s="8" t="n"/>
       <c r="AB21" s="8" t="inlineStr">
         <is>
@@ -2496,7 +2564,11 @@
       <c r="AU21" s="8" t="n"/>
       <c r="AV21" s="8" t="n"/>
       <c r="AW21" s="8" t="n"/>
-      <c r="AX21" s="8" t="n"/>
+      <c r="AX21" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n"/>
@@ -2515,7 +2587,7 @@
       <c r="F22" s="8" t="n"/>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Civil &amp; Sitework</t>
         </is>
       </c>
       <c r="H22" s="8" t="inlineStr">
@@ -2605,7 +2677,7 @@
       <c r="F23" s="8" t="n"/>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Civil &amp; Sitework</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
@@ -2695,7 +2767,7 @@
       <c r="F24" s="8" t="n"/>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Civil &amp; Sitework</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr">
@@ -2785,7 +2857,7 @@
       <c r="F25" s="8" t="n"/>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Civil &amp; Sitework</t>
         </is>
       </c>
       <c r="H25" s="8" t="inlineStr">
@@ -2875,7 +2947,7 @@
       <c r="F26" s="8" t="n"/>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Civil &amp; Sitework</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">
@@ -2970,7 +3042,7 @@
       </c>
       <c r="H27" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>Mild steel bar</t>
         </is>
       </c>
       <c r="I27" s="8" t="inlineStr">
@@ -2984,7 +3056,7 @@
         </is>
       </c>
       <c r="K27" s="17" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="L27" s="8" t="n"/>
       <c r="M27" s="8" t="n"/>
@@ -3007,8 +3079,12 @@
       <c r="V27" s="8" t="n"/>
       <c r="W27" s="8" t="n"/>
       <c r="X27" s="8" t="n"/>
-      <c r="Y27" s="8" t="n"/>
-      <c r="Z27" s="8" t="n"/>
+      <c r="Y27" s="17" t="n">
+        <v>155</v>
+      </c>
+      <c r="Z27" s="17" t="n">
+        <v>1.55</v>
+      </c>
       <c r="AA27" s="8" t="n"/>
       <c r="AB27" s="8" t="inlineStr">
         <is>
@@ -3036,7 +3112,11 @@
       <c r="AU27" s="8" t="n"/>
       <c r="AV27" s="8" t="n"/>
       <c r="AW27" s="8" t="n"/>
-      <c r="AX27" s="8" t="n"/>
+      <c r="AX27" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="n"/>
@@ -3060,7 +3140,7 @@
       </c>
       <c r="H28" s="8" t="inlineStr">
         <is>
-          <t>Cold twisted steel</t>
+          <t>Cold twisted bar</t>
         </is>
       </c>
       <c r="I28" s="8" t="inlineStr">
@@ -3074,7 +3154,7 @@
         </is>
       </c>
       <c r="K28" s="17" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="L28" s="8" t="n"/>
       <c r="M28" s="8" t="n"/>
@@ -3097,8 +3177,12 @@
       <c r="V28" s="8" t="n"/>
       <c r="W28" s="8" t="n"/>
       <c r="X28" s="8" t="n"/>
-      <c r="Y28" s="8" t="n"/>
-      <c r="Z28" s="8" t="n"/>
+      <c r="Y28" s="17" t="n">
+        <v>2131.25</v>
+      </c>
+      <c r="Z28" s="17" t="n">
+        <v>1.55</v>
+      </c>
       <c r="AA28" s="8" t="n"/>
       <c r="AB28" s="8" t="inlineStr">
         <is>
@@ -3126,7 +3210,11 @@
       <c r="AU28" s="8" t="n"/>
       <c r="AV28" s="8" t="n"/>
       <c r="AW28" s="8" t="n"/>
-      <c r="AX28" s="8" t="n"/>
+      <c r="AX28" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="n"/>
@@ -3155,7 +3243,7 @@
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
-          <t>Cement, Coarse sand, Graded stone aggregate</t>
+          <t>Cement, Coarse sand, Stone aggregate</t>
         </is>
       </c>
       <c r="J29" s="8" t="inlineStr">
@@ -3164,7 +3252,7 @@
         </is>
       </c>
       <c r="K29" s="17" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="L29" s="8" t="n"/>
       <c r="M29" s="8" t="inlineStr">
@@ -3191,8 +3279,12 @@
       <c r="V29" s="8" t="n"/>
       <c r="W29" s="8" t="n"/>
       <c r="X29" s="8" t="n"/>
-      <c r="Y29" s="8" t="n"/>
-      <c r="Z29" s="8" t="n"/>
+      <c r="Y29" s="17" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="Z29" s="17" t="n">
+        <v>0.149</v>
+      </c>
       <c r="AA29" s="8" t="n"/>
       <c r="AB29" s="8" t="inlineStr">
         <is>
@@ -3220,7 +3312,11 @@
       <c r="AU29" s="8" t="n"/>
       <c r="AV29" s="8" t="n"/>
       <c r="AW29" s="8" t="n"/>
-      <c r="AX29" s="8" t="n"/>
+      <c r="AX29" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="n"/>
@@ -3233,7 +3329,7 @@
       <c r="D30" s="8" t="n"/>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>Brick work with bricks of class designation___ in foundation and plinth in cement mortar 1:6 (1 cement : 6 coarse sand).</t>
+          <t>Brick work with bricks of class designation in foundation and plinth in cement mortar 1:6 (1 cement : 6 coarse sand).</t>
         </is>
       </c>
       <c r="F30" s="8" t="n"/>
@@ -3244,12 +3340,12 @@
       </c>
       <c r="H30" s="8" t="inlineStr">
         <is>
-          <t>Burnt brick</t>
+          <t>Brick work</t>
         </is>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
-          <t>Brick, Cement, Coarse sand</t>
+          <t>Brick, Cement, Sand</t>
         </is>
       </c>
       <c r="J30" s="8" t="inlineStr">
@@ -3285,12 +3381,16 @@
       <c r="V30" s="8" t="n"/>
       <c r="W30" s="8" t="n"/>
       <c r="X30" s="8" t="n"/>
-      <c r="Y30" s="8" t="n"/>
-      <c r="Z30" s="8" t="n"/>
+      <c r="Y30" s="17" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="Z30" s="17" t="n">
+        <v>0.213</v>
+      </c>
       <c r="AA30" s="8" t="n"/>
       <c r="AB30" s="8" t="inlineStr">
         <is>
-          <t>6.1.14/6.5.1 6.5.2</t>
+          <t>6.1.14/6.5.1/6.5.2</t>
         </is>
       </c>
       <c r="AC30" s="8" t="n"/>
@@ -3314,7 +3414,11 @@
       <c r="AU30" s="8" t="n"/>
       <c r="AV30" s="8" t="n"/>
       <c r="AW30" s="8" t="n"/>
-      <c r="AX30" s="8" t="n"/>
+      <c r="AX30" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Brick Clay) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="n"/>
@@ -3327,7 +3431,7 @@
       <c r="D31" s="8" t="n"/>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>Brick work with bricks of class designation___ in super structure above plinth upto floor two level in cement mortar 1:6 (1 cement : 6 coarse sand).</t>
+          <t>Brick work with bricks of class designation in super structure above plinth upto floor two level in cement mortar 1:6 (1 cement : 6 coarse sand).</t>
         </is>
       </c>
       <c r="F31" s="8" t="n"/>
@@ -3338,12 +3442,12 @@
       </c>
       <c r="H31" s="8" t="inlineStr">
         <is>
-          <t>Burnt brick</t>
+          <t>Brick work</t>
         </is>
       </c>
       <c r="I31" s="8" t="inlineStr">
         <is>
-          <t>Brick, Cement, Coarse sand</t>
+          <t>Brick, Cement, Sand</t>
         </is>
       </c>
       <c r="J31" s="8" t="inlineStr">
@@ -3379,12 +3483,16 @@
       <c r="V31" s="8" t="n"/>
       <c r="W31" s="8" t="n"/>
       <c r="X31" s="8" t="n"/>
-      <c r="Y31" s="8" t="n"/>
-      <c r="Z31" s="8" t="n"/>
+      <c r="Y31" s="17" t="n">
+        <v>8.58</v>
+      </c>
+      <c r="Z31" s="17" t="n">
+        <v>0.213</v>
+      </c>
       <c r="AA31" s="8" t="n"/>
       <c r="AB31" s="8" t="inlineStr">
         <is>
-          <t>6.1.14/6.3 6.5.1/6.5.2</t>
+          <t>6.1.14/6.3/6.5.1/6.5.2</t>
         </is>
       </c>
       <c r="AC31" s="8" t="n"/>
@@ -3408,7 +3516,11 @@
       <c r="AU31" s="8" t="n"/>
       <c r="AV31" s="8" t="n"/>
       <c r="AW31" s="8" t="n"/>
-      <c r="AX31" s="8" t="n"/>
+      <c r="AX31" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Brick Clay) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="n"/>
@@ -3421,7 +3533,7 @@
       <c r="D32" s="8" t="n"/>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>Brick work 7 cm thick with bricks of class designation ------ in super structure upto floor two level in cement mortar 1:3 (1 cement : 3 coarse sand).</t>
+          <t>Brick work 7 cm thick with bricks of class designation in super structure upto floor two level in cement mortar 1:3 (1 cement : 3 coarse sand).</t>
         </is>
       </c>
       <c r="F32" s="8" t="n"/>
@@ -3432,12 +3544,12 @@
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>Burnt brick</t>
+          <t>Brick work</t>
         </is>
       </c>
       <c r="I32" s="8" t="inlineStr">
         <is>
-          <t>Brick, Cement, Coarse sand</t>
+          <t>Brick, Cement, Sand</t>
         </is>
       </c>
       <c r="J32" s="8" t="inlineStr">
@@ -3473,12 +3585,16 @@
       <c r="V32" s="8" t="n"/>
       <c r="W32" s="8" t="n"/>
       <c r="X32" s="8" t="n"/>
-      <c r="Y32" s="8" t="n"/>
-      <c r="Z32" s="8" t="n"/>
+      <c r="Y32" s="17" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="Z32" s="17" t="n">
+        <v>0.213</v>
+      </c>
       <c r="AA32" s="8" t="n"/>
       <c r="AB32" s="8" t="inlineStr">
         <is>
-          <t>6.13/6.21/ 6.5.1/6.5.2</t>
+          <t>6.13/6.21/6.5.1/6.5.2</t>
         </is>
       </c>
       <c r="AC32" s="8" t="n"/>
@@ -3504,7 +3620,11 @@
       <c r="AU32" s="8" t="n"/>
       <c r="AV32" s="8" t="n"/>
       <c r="AW32" s="8" t="n"/>
-      <c r="AX32" s="8" t="n"/>
+      <c r="AX32" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Brick Clay) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="n"/>
@@ -3517,7 +3637,7 @@
       <c r="D33" s="8" t="n"/>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>Half brick masonry with bricks of class designation ____ in foundation &amp; plinth in cement mortar 1:4 (1 cement : 4 coarse sand)</t>
+          <t>Half brick masonry with bricks of class designation in foundation &amp; plinth in cement mortar 1:4 (1 cement : 4 coarse sand)</t>
         </is>
       </c>
       <c r="F33" s="8" t="n"/>
@@ -3528,12 +3648,12 @@
       </c>
       <c r="H33" s="8" t="inlineStr">
         <is>
-          <t>Burnt brick</t>
+          <t>Brick masonry</t>
         </is>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
-          <t>Brick, Cement, Coarse sand</t>
+          <t>Brick, Cement, Sand</t>
         </is>
       </c>
       <c r="J33" s="8" t="inlineStr">
@@ -3569,12 +3689,16 @@
       <c r="V33" s="8" t="n"/>
       <c r="W33" s="8" t="n"/>
       <c r="X33" s="8" t="n"/>
-      <c r="Y33" s="8" t="n"/>
-      <c r="Z33" s="8" t="n"/>
+      <c r="Y33" s="17" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="Z33" s="17" t="n">
+        <v>0.213</v>
+      </c>
       <c r="AA33" s="8" t="n"/>
       <c r="AB33" s="8" t="inlineStr">
         <is>
-          <t>6.18.4/6.21 6.5.1/6.5.2</t>
+          <t>6.18.4/6.21/6.5.1/6.5.2</t>
         </is>
       </c>
       <c r="AC33" s="8" t="n"/>
@@ -3598,7 +3722,11 @@
       <c r="AU33" s="8" t="n"/>
       <c r="AV33" s="8" t="n"/>
       <c r="AW33" s="8" t="n"/>
-      <c r="AX33" s="8" t="n"/>
+      <c r="AX33" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Brick Clay) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="n"/>
@@ -3611,7 +3739,7 @@
       <c r="D34" s="8" t="n"/>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>Half brick masonry with bricks of class designation ____ in super structure upto floor two level in cement mortar 1:4 (1 cement : 4 coarse sand).</t>
+          <t>Half brick masonry with bricks of class designation in super structure upto floor two level in cement mortar 1:4 (1 cement : 4 coarse sand).</t>
         </is>
       </c>
       <c r="F34" s="8" t="n"/>
@@ -3622,12 +3750,12 @@
       </c>
       <c r="H34" s="8" t="inlineStr">
         <is>
-          <t>Burnt brick</t>
+          <t>Brick masonry</t>
         </is>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
-          <t>Brick, Cement, Coarse sand</t>
+          <t>Brick, Cement, Sand</t>
         </is>
       </c>
       <c r="J34" s="8" t="inlineStr">
@@ -3663,12 +3791,16 @@
       <c r="V34" s="8" t="n"/>
       <c r="W34" s="8" t="n"/>
       <c r="X34" s="8" t="n"/>
-      <c r="Y34" s="8" t="n"/>
-      <c r="Z34" s="8" t="n"/>
+      <c r="Y34" s="17" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="Z34" s="17" t="n">
+        <v>0.213</v>
+      </c>
       <c r="AA34" s="8" t="n"/>
       <c r="AB34" s="8" t="inlineStr">
         <is>
-          <t>6.18.4/6.19.1 6.20/6.21.1/ 6.21.2</t>
+          <t>6.18.4/6.19.1/6.20/6.21.1/6.21.2</t>
         </is>
       </c>
       <c r="AC34" s="8" t="n"/>
@@ -3692,7 +3824,11 @@
       <c r="AU34" s="8" t="n"/>
       <c r="AV34" s="8" t="n"/>
       <c r="AW34" s="8" t="n"/>
-      <c r="AX34" s="8" t="n"/>
+      <c r="AX34" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Brick Clay) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="n"/>
@@ -3705,7 +3841,7 @@
       <c r="D35" s="8" t="n"/>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>Providing ________ wood work in frames of doors, windows, clerestory windows and other frames, wrought framed and fixed in position.</t>
+          <t>Providing wood work in frames of doors, windows, clerestory windows and other frames, wrought framed and fixed in position.</t>
         </is>
       </c>
       <c r="F35" s="8" t="n"/>
@@ -3716,7 +3852,7 @@
       </c>
       <c r="H35" s="8" t="inlineStr">
         <is>
-          <t>Wood</t>
+          <t>Wood work</t>
         </is>
       </c>
       <c r="I35" s="8" t="inlineStr">
@@ -3753,8 +3889,12 @@
       <c r="V35" s="8" t="n"/>
       <c r="W35" s="8" t="n"/>
       <c r="X35" s="8" t="n"/>
-      <c r="Y35" s="8" t="n"/>
-      <c r="Z35" s="8" t="n"/>
+      <c r="Y35" s="17" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="Z35" s="17" t="n">
+        <v>0.306</v>
+      </c>
       <c r="AA35" s="8" t="n"/>
       <c r="AB35" s="8" t="n"/>
       <c r="AC35" s="8" t="n"/>
@@ -3778,7 +3918,11 @@
       <c r="AU35" s="8" t="n"/>
       <c r="AV35" s="8" t="n"/>
       <c r="AW35" s="8" t="n"/>
-      <c r="AX35" s="8" t="n"/>
+      <c r="AX35" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Timber Hardwood) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="n"/>
@@ -3791,7 +3935,7 @@
       <c r="D36" s="8" t="n"/>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t>Providing and fixing 35 mm thick battened and framed door shutters of ________ wood including bright finished or/and black enamelled MS butt hinges with necessary screws.</t>
+          <t>Providing and fixing 35 mm thick battended and framed door shutters of wood including bright finished or/and black enamelled MS butt hinges with necessary screws.</t>
         </is>
       </c>
       <c r="F36" s="8" t="n"/>
@@ -3802,12 +3946,12 @@
       </c>
       <c r="H36" s="8" t="inlineStr">
         <is>
-          <t>Wood</t>
+          <t>Wood door shutters</t>
         </is>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
-          <t>Wood, Mild steel</t>
+          <t>Wood, MS butt hinges</t>
         </is>
       </c>
       <c r="J36" s="8" t="inlineStr">
@@ -3839,8 +3983,12 @@
       <c r="V36" s="8" t="n"/>
       <c r="W36" s="8" t="n"/>
       <c r="X36" s="8" t="n"/>
-      <c r="Y36" s="8" t="n"/>
-      <c r="Z36" s="8" t="n"/>
+      <c r="Y36" s="17" t="n">
+        <v>5.51</v>
+      </c>
+      <c r="Z36" s="17" t="n">
+        <v>0.306</v>
+      </c>
       <c r="AA36" s="8" t="n"/>
       <c r="AB36" s="8" t="n"/>
       <c r="AC36" s="8" t="n"/>
@@ -3866,7 +4014,11 @@
       <c r="AU36" s="8" t="n"/>
       <c r="AV36" s="8" t="n"/>
       <c r="AW36" s="8" t="n"/>
-      <c r="AX36" s="8" t="n"/>
+      <c r="AX36" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Timber Hardwood) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="n"/>
@@ -3890,12 +4042,12 @@
       </c>
       <c r="H37" s="8" t="inlineStr">
         <is>
-          <t>Flush door</t>
+          <t>Flush door shutter</t>
         </is>
       </c>
       <c r="I37" s="8" t="inlineStr">
         <is>
-          <t>Hard wood, Teak ply, Commercial ply, Mild steel</t>
+          <t>Block board, Hard wood, Teak ply, Commercial ply, MS piano hinges</t>
         </is>
       </c>
       <c r="J37" s="8" t="inlineStr">
@@ -3927,8 +4079,12 @@
       <c r="V37" s="8" t="n"/>
       <c r="W37" s="8" t="n"/>
       <c r="X37" s="8" t="n"/>
-      <c r="Y37" s="8" t="n"/>
-      <c r="Z37" s="8" t="n"/>
+      <c r="Y37" s="17" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="Z37" s="17" t="n">
+        <v>0.306</v>
+      </c>
       <c r="AA37" s="8" t="n"/>
       <c r="AB37" s="8" t="inlineStr">
         <is>
@@ -3958,7 +4114,11 @@
       <c r="AU37" s="8" t="n"/>
       <c r="AV37" s="8" t="n"/>
       <c r="AW37" s="8" t="n"/>
-      <c r="AX37" s="8" t="n"/>
+      <c r="AX37" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Timber Hardwood) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n"/>
@@ -3977,12 +4137,12 @@
       <c r="F38" s="8" t="n"/>
       <c r="G38" s="8" t="inlineStr">
         <is>
-          <t>Finishes</t>
+          <t>Civil &amp; Sitework</t>
         </is>
       </c>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t>Teak wood</t>
+          <t>Teak wood plugs</t>
         </is>
       </c>
       <c r="I38" s="8" t="inlineStr">
@@ -4023,8 +4183,12 @@
       <c r="V38" s="8" t="n"/>
       <c r="W38" s="8" t="n"/>
       <c r="X38" s="8" t="n"/>
-      <c r="Y38" s="8" t="n"/>
-      <c r="Z38" s="8" t="n"/>
+      <c r="Y38" s="17" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="Z38" s="17" t="n">
+        <v>0.306</v>
+      </c>
       <c r="AA38" s="8" t="n"/>
       <c r="AB38" s="8" t="inlineStr">
         <is>
@@ -4052,7 +4216,11 @@
       <c r="AU38" s="8" t="n"/>
       <c r="AV38" s="8" t="n"/>
       <c r="AW38" s="8" t="n"/>
-      <c r="AX38" s="8" t="n"/>
+      <c r="AX38" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Timber Hardwood) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="n"/>
@@ -4065,7 +4233,7 @@
       <c r="D39" s="8" t="n"/>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>Providing and fixing M.S.oxidised fan light .ventilator catch with necessary screws etc. complete.</t>
+          <t>Providing and fixing M.S.oxidised fan light ventilator catch with necessary screws etc. complete.</t>
         </is>
       </c>
       <c r="F39" s="8" t="n"/>
@@ -4076,12 +4244,12 @@
       </c>
       <c r="H39" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>M.S. oxidised fan light ventilator catch</t>
         </is>
       </c>
       <c r="I39" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>M.S.</t>
         </is>
       </c>
       <c r="J39" s="8" t="inlineStr">
@@ -4090,7 +4258,7 @@
         </is>
       </c>
       <c r="K39" s="17" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="L39" s="8" t="n"/>
       <c r="M39" s="8" t="n"/>
@@ -4113,8 +4281,12 @@
       <c r="V39" s="8" t="n"/>
       <c r="W39" s="8" t="n"/>
       <c r="X39" s="8" t="n"/>
-      <c r="Y39" s="8" t="n"/>
-      <c r="Z39" s="8" t="n"/>
+      <c r="Y39" s="17" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="Z39" s="17" t="n">
+        <v>1.55</v>
+      </c>
       <c r="AA39" s="8" t="n"/>
       <c r="AB39" s="8" t="n"/>
       <c r="AC39" s="8" t="n"/>
@@ -4138,7 +4310,11 @@
       <c r="AU39" s="8" t="n"/>
       <c r="AV39" s="8" t="n"/>
       <c r="AW39" s="8" t="n"/>
-      <c r="AX39" s="8" t="n"/>
+      <c r="AX39" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="n"/>
@@ -4151,7 +4327,7 @@
       <c r="D40" s="8" t="n"/>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t>Providing and fixing 90 mm oxidised M.S. hasp and staple (safety type) with necessaary screws etc. complete.</t>
+          <t>Providing and fixing 90 mm oxidised M.S. hasp and staple (safety type) with necessary screws etc. complete.</t>
         </is>
       </c>
       <c r="F40" s="8" t="n"/>
@@ -4162,12 +4338,12 @@
       </c>
       <c r="H40" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>Oxidised M.S. hasp and staple</t>
         </is>
       </c>
       <c r="I40" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>M.S.</t>
         </is>
       </c>
       <c r="J40" s="8" t="inlineStr">
@@ -4176,7 +4352,7 @@
         </is>
       </c>
       <c r="K40" s="17" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="L40" s="8" t="n"/>
       <c r="M40" s="8" t="n"/>
@@ -4199,8 +4375,12 @@
       <c r="V40" s="8" t="n"/>
       <c r="W40" s="8" t="n"/>
       <c r="X40" s="8" t="n"/>
-      <c r="Y40" s="8" t="n"/>
-      <c r="Z40" s="8" t="n"/>
+      <c r="Y40" s="17" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Z40" s="17" t="n">
+        <v>1.55</v>
+      </c>
       <c r="AA40" s="8" t="n"/>
       <c r="AB40" s="8" t="inlineStr">
         <is>
@@ -4228,7 +4408,11 @@
       <c r="AU40" s="8" t="n"/>
       <c r="AV40" s="8" t="n"/>
       <c r="AW40" s="8" t="n"/>
-      <c r="AX40" s="8" t="n"/>
+      <c r="AX40" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="n"/>
@@ -4252,7 +4436,7 @@
       </c>
       <c r="H41" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium sliding door bolts</t>
         </is>
       </c>
       <c r="I41" s="8" t="inlineStr">
@@ -4344,7 +4528,7 @@
       </c>
       <c r="H42" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium tower bolts</t>
         </is>
       </c>
       <c r="I42" s="8" t="inlineStr">
@@ -4436,7 +4620,7 @@
       </c>
       <c r="H43" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium tower bolts</t>
         </is>
       </c>
       <c r="I43" s="8" t="inlineStr">
@@ -4528,7 +4712,7 @@
       </c>
       <c r="H44" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium handles</t>
         </is>
       </c>
       <c r="I44" s="8" t="inlineStr">
@@ -4618,7 +4802,7 @@
       </c>
       <c r="H45" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium handles</t>
         </is>
       </c>
       <c r="I45" s="8" t="inlineStr">
@@ -4708,7 +4892,7 @@
       </c>
       <c r="H46" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium door stopper</t>
         </is>
       </c>
       <c r="I46" s="8" t="inlineStr">
@@ -4798,12 +4982,12 @@
       </c>
       <c r="H47" s="8" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>Steel glazed windows</t>
         </is>
       </c>
       <c r="I47" s="8" t="inlineStr">
         <is>
-          <t>Steel, Cement, Coarse sand, Graded stone aggregate, Glass</t>
+          <t>Steel, Cement, Coarse sand, Stone aggregate, Glass, Putty</t>
         </is>
       </c>
       <c r="J47" s="8" t="inlineStr">
@@ -4839,8 +5023,12 @@
       <c r="V47" s="8" t="n"/>
       <c r="W47" s="8" t="n"/>
       <c r="X47" s="8" t="n"/>
-      <c r="Y47" s="8" t="n"/>
-      <c r="Z47" s="8" t="n"/>
+      <c r="Y47" s="17" t="n">
+        <v>17.52</v>
+      </c>
+      <c r="Z47" s="17" t="n">
+        <v>1.55</v>
+      </c>
       <c r="AA47" s="8" t="n"/>
       <c r="AB47" s="8" t="inlineStr">
         <is>
@@ -4870,7 +5058,11 @@
       <c r="AU47" s="8" t="n"/>
       <c r="AV47" s="8" t="n"/>
       <c r="AW47" s="8" t="n"/>
-      <c r="AX47" s="8" t="n"/>
+      <c r="AX47" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="8" t="n"/>
@@ -4894,12 +5086,12 @@
       </c>
       <c r="H48" s="8" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>Steel glazed ventilators</t>
         </is>
       </c>
       <c r="I48" s="8" t="inlineStr">
         <is>
-          <t>Steel, Cement, Coarse sand, Graded stone aggregate, Glass</t>
+          <t>Steel, Cement, Coarse sand, Stone aggregate, Glass, Putty</t>
         </is>
       </c>
       <c r="J48" s="8" t="inlineStr">
@@ -4935,8 +5127,12 @@
       <c r="V48" s="8" t="n"/>
       <c r="W48" s="8" t="n"/>
       <c r="X48" s="8" t="n"/>
-      <c r="Y48" s="8" t="n"/>
-      <c r="Z48" s="8" t="n"/>
+      <c r="Y48" s="17" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="Z48" s="17" t="n">
+        <v>1.55</v>
+      </c>
       <c r="AA48" s="8" t="n"/>
       <c r="AB48" s="8" t="inlineStr">
         <is>
@@ -4966,7 +5162,11 @@
       <c r="AU48" s="8" t="n"/>
       <c r="AV48" s="8" t="n"/>
       <c r="AW48" s="8" t="n"/>
-      <c r="AX48" s="8" t="n"/>
+      <c r="AX48" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="n"/>
@@ -4990,7 +5190,7 @@
       </c>
       <c r="H49" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>Mild steel casement window fastners</t>
         </is>
       </c>
       <c r="I49" s="8" t="inlineStr">
@@ -5027,8 +5227,12 @@
       <c r="V49" s="8" t="n"/>
       <c r="W49" s="8" t="n"/>
       <c r="X49" s="8" t="n"/>
-      <c r="Y49" s="8" t="n"/>
-      <c r="Z49" s="8" t="n"/>
+      <c r="Y49" s="17" t="n">
+        <v>32.55</v>
+      </c>
+      <c r="Z49" s="17" t="n">
+        <v>1.55</v>
+      </c>
       <c r="AA49" s="8" t="n"/>
       <c r="AB49" s="8" t="inlineStr">
         <is>
@@ -5056,7 +5260,11 @@
       <c r="AU49" s="8" t="n"/>
       <c r="AV49" s="8" t="n"/>
       <c r="AW49" s="8" t="n"/>
-      <c r="AX49" s="8" t="n"/>
+      <c r="AX49" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="n"/>
@@ -5069,7 +5277,7 @@
       <c r="D50" s="8" t="n"/>
       <c r="E50" s="8" t="inlineStr">
         <is>
-          <t>Providing and fixing aluminium casement stays anodised transparent or dyed to requird colour and shade with with necessary welding and machine screws etc. complete.</t>
+          <t>Providing and fixing aluminium casement stays anodised transparent or dyed to required colour and shade with with necessary welding and machine screws etc. complete.</t>
         </is>
       </c>
       <c r="F50" s="8" t="n"/>
@@ -5080,7 +5288,7 @@
       </c>
       <c r="H50" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium casement stays</t>
         </is>
       </c>
       <c r="I50" s="8" t="inlineStr">
@@ -5170,12 +5378,12 @@
       </c>
       <c r="H51" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>M S Guard Flats</t>
         </is>
       </c>
       <c r="I51" s="8" t="inlineStr">
         <is>
-          <t>Mild steel, Steel primer</t>
+          <t>MS, Steel primer</t>
         </is>
       </c>
       <c r="J51" s="8" t="inlineStr">
@@ -5207,8 +5415,12 @@
       <c r="V51" s="8" t="n"/>
       <c r="W51" s="8" t="n"/>
       <c r="X51" s="8" t="n"/>
-      <c r="Y51" s="8" t="n"/>
-      <c r="Z51" s="8" t="n"/>
+      <c r="Y51" s="17" t="n">
+        <v>102.3</v>
+      </c>
+      <c r="Z51" s="17" t="n">
+        <v>1.55</v>
+      </c>
       <c r="AA51" s="8" t="n"/>
       <c r="AB51" s="8" t="inlineStr">
         <is>
@@ -5238,7 +5450,11 @@
       <c r="AU51" s="8" t="n"/>
       <c r="AV51" s="8" t="n"/>
       <c r="AW51" s="8" t="n"/>
-      <c r="AX51" s="8" t="n"/>
+      <c r="AX51" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="8" t="n"/>
@@ -5262,12 +5478,12 @@
       </c>
       <c r="H52" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>T-Iron frames</t>
         </is>
       </c>
       <c r="I52" s="8" t="inlineStr">
         <is>
-          <t>Mild steel, Cement, Coarse sand, Graded stone aggregate</t>
+          <t>Mild steel, Cement, Sand, Stone aggregate, Steel primer</t>
         </is>
       </c>
       <c r="J52" s="8" t="inlineStr">
@@ -5303,8 +5519,12 @@
       <c r="V52" s="8" t="n"/>
       <c r="W52" s="8" t="n"/>
       <c r="X52" s="8" t="n"/>
-      <c r="Y52" s="8" t="n"/>
-      <c r="Z52" s="8" t="n"/>
+      <c r="Y52" s="17" t="n">
+        <v>289.85</v>
+      </c>
+      <c r="Z52" s="17" t="n">
+        <v>1.55</v>
+      </c>
       <c r="AA52" s="8" t="n"/>
       <c r="AB52" s="8" t="inlineStr">
         <is>
@@ -5332,7 +5552,11 @@
       <c r="AU52" s="8" t="n"/>
       <c r="AV52" s="8" t="n"/>
       <c r="AW52" s="8" t="n"/>
-      <c r="AX52" s="8" t="n"/>
+      <c r="AX52" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="n"/>
@@ -5356,12 +5580,12 @@
       </c>
       <c r="H53" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>MS fan clamp</t>
         </is>
       </c>
       <c r="I53" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>MS bar, Paint</t>
         </is>
       </c>
       <c r="J53" s="8" t="inlineStr">
@@ -5393,8 +5617,12 @@
       <c r="V53" s="8" t="n"/>
       <c r="W53" s="8" t="n"/>
       <c r="X53" s="8" t="n"/>
-      <c r="Y53" s="8" t="n"/>
-      <c r="Z53" s="8" t="n"/>
+      <c r="Y53" s="17" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="Z53" s="17" t="n">
+        <v>1.55</v>
+      </c>
       <c r="AA53" s="8" t="n"/>
       <c r="AB53" s="8" t="inlineStr">
         <is>
@@ -5424,7 +5652,11 @@
       <c r="AU53" s="8" t="n"/>
       <c r="AV53" s="8" t="n"/>
       <c r="AW53" s="8" t="n"/>
-      <c r="AX53" s="8" t="n"/>
+      <c r="AX53" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="n"/>
@@ -5448,12 +5680,12 @@
       </c>
       <c r="H54" s="8" t="inlineStr">
         <is>
-          <t>Cement concrete</t>
+          <t>Cement concrete flooring</t>
         </is>
       </c>
       <c r="I54" s="8" t="inlineStr">
         <is>
-          <t>Cement, Coarse sand, Graded stone aggregate</t>
+          <t>Cement, Coarse sand, Stone aggregate</t>
         </is>
       </c>
       <c r="J54" s="8" t="inlineStr">
@@ -5462,7 +5694,7 @@
         </is>
       </c>
       <c r="K54" s="17" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="L54" s="8" t="n"/>
       <c r="M54" s="8" t="inlineStr">
@@ -5489,8 +5721,12 @@
       <c r="V54" s="8" t="n"/>
       <c r="W54" s="8" t="n"/>
       <c r="X54" s="8" t="n"/>
-      <c r="Y54" s="8" t="n"/>
-      <c r="Z54" s="8" t="n"/>
+      <c r="Y54" s="17" t="n">
+        <v>10.13</v>
+      </c>
+      <c r="Z54" s="17" t="n">
+        <v>0.149</v>
+      </c>
       <c r="AA54" s="8" t="n"/>
       <c r="AB54" s="8" t="inlineStr">
         <is>
@@ -5520,7 +5756,11 @@
       <c r="AU54" s="8" t="n"/>
       <c r="AV54" s="8" t="n"/>
       <c r="AW54" s="8" t="n"/>
-      <c r="AX54" s="8" t="n"/>
+      <c r="AX54" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="n"/>
@@ -5544,7 +5784,7 @@
       </c>
       <c r="H55" s="8" t="inlineStr">
         <is>
-          <t>Cement plaster</t>
+          <t>Cement plaster skirting</t>
         </is>
       </c>
       <c r="I55" s="8" t="inlineStr">
@@ -5585,8 +5825,12 @@
       <c r="V55" s="8" t="n"/>
       <c r="W55" s="8" t="n"/>
       <c r="X55" s="8" t="n"/>
-      <c r="Y55" s="8" t="n"/>
-      <c r="Z55" s="8" t="n"/>
+      <c r="Y55" s="17" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="Z55" s="17" t="n">
+        <v>0.95</v>
+      </c>
       <c r="AA55" s="8" t="n"/>
       <c r="AB55" s="8" t="inlineStr">
         <is>
@@ -5616,7 +5860,11 @@
       <c r="AU55" s="8" t="n"/>
       <c r="AV55" s="8" t="n"/>
       <c r="AW55" s="8" t="n"/>
-      <c r="AX55" s="8" t="n"/>
+      <c r="AX55" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V3.0 (Generic Assumed)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="8" t="n"/>
@@ -5640,17 +5888,17 @@
       </c>
       <c r="H56" s="8" t="inlineStr">
         <is>
-          <t>Marble chips</t>
+          <t>Marble chips flooring</t>
         </is>
       </c>
       <c r="I56" s="8" t="inlineStr">
         <is>
-          <t>Cement, Coarse sand, Graded stone aggregate, Marble chips, Marble powder</t>
+          <t>Cement, Sand, Stone aggregate, Marble chips, Marble powder, Pigment</t>
         </is>
       </c>
       <c r="J56" s="8" t="inlineStr">
         <is>
-          <t>Paint/Finish</t>
+          <t>Finishes</t>
         </is>
       </c>
       <c r="K56" s="17" t="n">
@@ -5736,21 +5984,21 @@
       </c>
       <c r="H57" s="8" t="inlineStr">
         <is>
+          <t>Glass strips</t>
+        </is>
+      </c>
+      <c r="I57" s="8" t="inlineStr">
+        <is>
           <t>Glass</t>
         </is>
       </c>
-      <c r="I57" s="8" t="inlineStr">
-        <is>
-          <t>Glass</t>
-        </is>
-      </c>
       <c r="J57" s="8" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
       <c r="K57" s="17" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="L57" s="8" t="n"/>
       <c r="M57" s="8" t="n"/>
@@ -5817,13 +6065,13 @@
       <c r="D58" s="8" t="n"/>
       <c r="E58" s="8" t="inlineStr">
         <is>
-          <t>Painting top of roofs with bitumen of approved quality at 17 Kg. per 10 square metre impregnated with a coat of coarse sand at 3/2 60 dm per 10 m including cleaning the slab surface with brushes and finally with a piece of cloth lightly soaked in kerosene oil complete with residual type petroleum bitumen of penetration 80/100.</t>
+          <t>Painting top of roofs with bitumen of approved quality at 17 Kg. per 10 square metre impregnated with a coat of coarse sand at 3/60 dm3 per 10 m2 including cleaning the slab surface with brushes and finally with a piece of cloth lightly soaked in kerosene oil complete with residual type petroleum bitumen of penetration 80/100.</t>
         </is>
       </c>
       <c r="F58" s="8" t="n"/>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>Finishes</t>
+          <t>Civil &amp; Sitework</t>
         </is>
       </c>
       <c r="H58" s="8" t="inlineStr">
@@ -5842,7 +6090,7 @@
         </is>
       </c>
       <c r="K58" s="17" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="L58" s="8" t="n"/>
       <c r="M58" s="8" t="n"/>
@@ -5865,8 +6113,12 @@
       <c r="V58" s="8" t="n"/>
       <c r="W58" s="8" t="n"/>
       <c r="X58" s="8" t="n"/>
-      <c r="Y58" s="8" t="n"/>
-      <c r="Z58" s="8" t="n"/>
+      <c r="Y58" s="17" t="n">
+        <v>61.75</v>
+      </c>
+      <c r="Z58" s="17" t="n">
+        <v>0.95</v>
+      </c>
       <c r="AA58" s="8" t="n"/>
       <c r="AB58" s="8" t="inlineStr">
         <is>
@@ -5894,7 +6146,11 @@
       <c r="AU58" s="8" t="n"/>
       <c r="AV58" s="8" t="n"/>
       <c r="AW58" s="8" t="n"/>
-      <c r="AX58" s="8" t="n"/>
+      <c r="AX58" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V3.0 (Generic Assumed)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="n"/>
@@ -5913,17 +6169,17 @@
       <c r="F59" s="8" t="n"/>
       <c r="G59" s="8" t="inlineStr">
         <is>
-          <t>Finishes</t>
+          <t>Civil &amp; Sitework</t>
         </is>
       </c>
       <c r="H59" s="8" t="inlineStr">
         <is>
-          <t>Lime concrete</t>
+          <t>Lime concrete terracing</t>
         </is>
       </c>
       <c r="I59" s="8" t="inlineStr">
         <is>
-          <t>Lime, Brick aggregate, Surkhi, Brick tiles, Cement, Fine sand, Crude oil</t>
+          <t>Brick aggregate, Lime putty, Surkhi, Gur, Belgiri, Brick tiles, Cement, Fine sand, Crude oil</t>
         </is>
       </c>
       <c r="J59" s="8" t="inlineStr">
@@ -5959,8 +6215,12 @@
       <c r="V59" s="8" t="n"/>
       <c r="W59" s="8" t="n"/>
       <c r="X59" s="8" t="n"/>
-      <c r="Y59" s="8" t="n"/>
-      <c r="Z59" s="8" t="n"/>
+      <c r="Y59" s="17" t="n">
+        <v>9.68</v>
+      </c>
+      <c r="Z59" s="17" t="n">
+        <v>0.149</v>
+      </c>
       <c r="AA59" s="8" t="n"/>
       <c r="AB59" s="8" t="inlineStr">
         <is>
@@ -5990,7 +6250,11 @@
       <c r="AU59" s="8" t="n"/>
       <c r="AV59" s="8" t="n"/>
       <c r="AW59" s="8" t="n"/>
-      <c r="AX59" s="8" t="n"/>
+      <c r="AX59" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="8" t="n"/>
@@ -6014,12 +6278,12 @@
       </c>
       <c r="H60" s="8" t="inlineStr">
         <is>
-          <t>Burnt clay tile</t>
+          <t>Burnt clay tiles</t>
         </is>
       </c>
       <c r="I60" s="8" t="inlineStr">
         <is>
-          <t>Burnt clay tile, Cement, Fine sand</t>
+          <t>Clay tiles, Cement, Fine sand</t>
         </is>
       </c>
       <c r="J60" s="8" t="inlineStr">
@@ -6055,8 +6319,12 @@
       <c r="V60" s="8" t="n"/>
       <c r="W60" s="8" t="n"/>
       <c r="X60" s="8" t="n"/>
-      <c r="Y60" s="8" t="n"/>
-      <c r="Z60" s="8" t="n"/>
+      <c r="Y60" s="17" t="n">
+        <v>6.82</v>
+      </c>
+      <c r="Z60" s="17" t="n">
+        <v>0.213</v>
+      </c>
       <c r="AA60" s="8" t="n"/>
       <c r="AB60" s="8" t="inlineStr">
         <is>
@@ -6086,7 +6354,11 @@
       <c r="AU60" s="8" t="n"/>
       <c r="AV60" s="8" t="n"/>
       <c r="AW60" s="8" t="n"/>
-      <c r="AX60" s="8" t="n"/>
+      <c r="AX60" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Brick Clay) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="n"/>
@@ -6110,12 +6382,12 @@
       </c>
       <c r="H61" s="8" t="inlineStr">
         <is>
-          <t>Cement concrete</t>
+          <t>Cement concrete gola</t>
         </is>
       </c>
       <c r="I61" s="8" t="inlineStr">
         <is>
-          <t>Cement, Coarse sand, Graded stone aggregate, Brick tile</t>
+          <t>Cement, Coarse sand, Stone aggregate, Brick tiles</t>
         </is>
       </c>
       <c r="J61" s="8" t="inlineStr">
@@ -6151,8 +6423,12 @@
       <c r="V61" s="8" t="n"/>
       <c r="W61" s="8" t="n"/>
       <c r="X61" s="8" t="n"/>
-      <c r="Y61" s="8" t="n"/>
-      <c r="Z61" s="8" t="n"/>
+      <c r="Y61" s="17" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="Z61" s="17" t="n">
+        <v>0.149</v>
+      </c>
       <c r="AA61" s="8" t="n"/>
       <c r="AB61" s="8" t="inlineStr">
         <is>
@@ -6180,7 +6456,11 @@
       <c r="AU61" s="8" t="n"/>
       <c r="AV61" s="8" t="n"/>
       <c r="AW61" s="8" t="n"/>
-      <c r="AX61" s="8" t="n"/>
+      <c r="AX61" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="8" t="n"/>
@@ -6204,12 +6484,12 @@
       </c>
       <c r="H62" s="8" t="inlineStr">
         <is>
-          <t>Cement concrete</t>
+          <t>Cement concrete khurras</t>
         </is>
       </c>
       <c r="I62" s="8" t="inlineStr">
         <is>
-          <t>Cement, Coarse sand, Graded stone aggregate, PVC sheet</t>
+          <t>Cement, Coarse sand, Stone aggregate, PVC sheet</t>
         </is>
       </c>
       <c r="J62" s="8" t="inlineStr">
@@ -6245,8 +6525,12 @@
       <c r="V62" s="8" t="n"/>
       <c r="W62" s="8" t="n"/>
       <c r="X62" s="8" t="n"/>
-      <c r="Y62" s="8" t="n"/>
-      <c r="Z62" s="8" t="n"/>
+      <c r="Y62" s="17" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="Z62" s="17" t="n">
+        <v>0.149</v>
+      </c>
       <c r="AA62" s="8" t="n"/>
       <c r="AB62" s="8" t="inlineStr">
         <is>
@@ -6276,7 +6560,11 @@
       <c r="AU62" s="8" t="n"/>
       <c r="AV62" s="8" t="n"/>
       <c r="AW62" s="8" t="n"/>
-      <c r="AX62" s="8" t="n"/>
+      <c r="AX62" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="n"/>
@@ -6300,12 +6588,12 @@
       </c>
       <c r="H63" s="8" t="inlineStr">
         <is>
-          <t>Cast iron</t>
+          <t>CI rain water pipe</t>
         </is>
       </c>
       <c r="I63" s="8" t="inlineStr">
         <is>
-          <t>Cast iron, Cement, Fine sand</t>
+          <t>Cast Iron, Spun yarn, Cement, Fine sand</t>
         </is>
       </c>
       <c r="J63" s="8" t="inlineStr">
@@ -6396,12 +6684,12 @@
       </c>
       <c r="H64" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>MS holderbat clamps</t>
         </is>
       </c>
       <c r="I64" s="8" t="inlineStr">
         <is>
-          <t>Mild steel, Cement, Coarse sand, Graded stone aggregate</t>
+          <t>MS, Cement, Coarse sand, Stone aggregate</t>
         </is>
       </c>
       <c r="J64" s="8" t="inlineStr">
@@ -6437,8 +6725,12 @@
       <c r="V64" s="8" t="n"/>
       <c r="W64" s="8" t="n"/>
       <c r="X64" s="8" t="n"/>
-      <c r="Y64" s="8" t="n"/>
-      <c r="Z64" s="8" t="n"/>
+      <c r="Y64" s="17" t="n">
+        <v>13.95</v>
+      </c>
+      <c r="Z64" s="17" t="n">
+        <v>1.55</v>
+      </c>
       <c r="AA64" s="8" t="n"/>
       <c r="AB64" s="8" t="inlineStr">
         <is>
@@ -6468,7 +6760,11 @@
       <c r="AU64" s="8" t="n"/>
       <c r="AV64" s="8" t="n"/>
       <c r="AW64" s="8" t="n"/>
-      <c r="AX64" s="8" t="n"/>
+      <c r="AX64" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="n"/>
@@ -6481,7 +6777,7 @@
       <c r="D65" s="8" t="n"/>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>Providing and fixing on wall face CI accessories for rain water pipes including filling the joints with spun yarn soaked in neat cement slurry and cement mortar 1:2 (1 cement : 2 fine sand). CI plain head 100 mm dia</t>
+          <t>Providing and fixing on wall face CI accessories for rain water pipes including filling the joints with spun yarn soaked in neat cement slurry and cement mortar 1:2 (1 cement : 2 fine sand) CI plain head 100 mm dia</t>
         </is>
       </c>
       <c r="F65" s="8" t="n"/>
@@ -6492,12 +6788,12 @@
       </c>
       <c r="H65" s="8" t="inlineStr">
         <is>
-          <t>Cast iron</t>
+          <t>CI plain head</t>
         </is>
       </c>
       <c r="I65" s="8" t="inlineStr">
         <is>
-          <t>Cast iron, Cement, Fine sand</t>
+          <t>Cast Iron, Spun yarn, Cement, Fine sand</t>
         </is>
       </c>
       <c r="J65" s="8" t="inlineStr">
@@ -6577,7 +6873,7 @@
       <c r="D66" s="8" t="n"/>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t>Providing and fixing on wall face CI accessories for rain water pipes including filling the joints with spun yarn soaked in neat cement slurry and cement mortar 1:2 (1 cement : 2 fine sand). CI plain shoe - 100 mm dia</t>
+          <t>Providing and fixing on wall face CI accessories for rain water pipes including filling the joints with spun yarn soaked in neat cement slurry and cement mortar 1:2 (1 cement : 2 fine sand) CI plain shoe - 100 mm dia</t>
         </is>
       </c>
       <c r="F66" s="8" t="n"/>
@@ -6588,12 +6884,12 @@
       </c>
       <c r="H66" s="8" t="inlineStr">
         <is>
-          <t>Cast iron</t>
+          <t>CI plain shoe</t>
         </is>
       </c>
       <c r="I66" s="8" t="inlineStr">
         <is>
-          <t>Cast iron, Cement, Fine sand</t>
+          <t>Cast Iron, Spun yarn, Cement, Fine sand</t>
         </is>
       </c>
       <c r="J66" s="8" t="inlineStr">
@@ -6673,7 +6969,7 @@
       <c r="D67" s="8" t="n"/>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t>Providing and fixing on wall face CI accessories for rain water pipes including filling the joints with spun yarn soaked in neat cement slurry and cement mortar 1:2 (1 cement : 2 fine sand). CI plain bend - 100 mm dia</t>
+          <t>Providing and fixing on wall face CI accessories for rain water pipes including filling the joints with spun yarn soaked in neat cement slurry and cement mortar 1:2 (1 cement : 2 fine sand) CI plain bend - 100 mm dia</t>
         </is>
       </c>
       <c r="F67" s="8" t="n"/>
@@ -6684,12 +6980,12 @@
       </c>
       <c r="H67" s="8" t="inlineStr">
         <is>
-          <t>Cast iron</t>
+          <t>CI plain bend</t>
         </is>
       </c>
       <c r="I67" s="8" t="inlineStr">
         <is>
-          <t>Cast iron, Cement, Fine sand</t>
+          <t>Cast Iron, Spun yarn, Cement, Fine sand</t>
         </is>
       </c>
       <c r="J67" s="8" t="inlineStr">
@@ -6821,8 +7117,12 @@
       <c r="V68" s="8" t="n"/>
       <c r="W68" s="8" t="n"/>
       <c r="X68" s="8" t="n"/>
-      <c r="Y68" s="8" t="n"/>
-      <c r="Z68" s="8" t="n"/>
+      <c r="Y68" s="17" t="n">
+        <v>209</v>
+      </c>
+      <c r="Z68" s="17" t="n">
+        <v>0.95</v>
+      </c>
       <c r="AA68" s="8" t="n"/>
       <c r="AB68" s="8" t="inlineStr">
         <is>
@@ -6852,7 +7152,11 @@
       <c r="AU68" s="8" t="n"/>
       <c r="AV68" s="8" t="n"/>
       <c r="AW68" s="8" t="n"/>
-      <c r="AX68" s="8" t="n"/>
+      <c r="AX68" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V3.0 (Generic Assumed)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="n"/>
@@ -6917,8 +7221,12 @@
       <c r="V69" s="8" t="n"/>
       <c r="W69" s="8" t="n"/>
       <c r="X69" s="8" t="n"/>
-      <c r="Y69" s="8" t="n"/>
-      <c r="Z69" s="8" t="n"/>
+      <c r="Y69" s="17" t="n">
+        <v>209</v>
+      </c>
+      <c r="Z69" s="17" t="n">
+        <v>0.95</v>
+      </c>
       <c r="AA69" s="8" t="n"/>
       <c r="AB69" s="8" t="inlineStr">
         <is>
@@ -6948,7 +7256,11 @@
       <c r="AU69" s="8" t="n"/>
       <c r="AV69" s="8" t="n"/>
       <c r="AW69" s="8" t="n"/>
-      <c r="AX69" s="8" t="n"/>
+      <c r="AX69" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V3.0 (Generic Assumed)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="8" t="n"/>
@@ -7013,8 +7325,12 @@
       <c r="V70" s="8" t="n"/>
       <c r="W70" s="8" t="n"/>
       <c r="X70" s="8" t="n"/>
-      <c r="Y70" s="8" t="n"/>
-      <c r="Z70" s="8" t="n"/>
+      <c r="Y70" s="17" t="n">
+        <v>18.05</v>
+      </c>
+      <c r="Z70" s="17" t="n">
+        <v>0.95</v>
+      </c>
       <c r="AA70" s="8" t="n"/>
       <c r="AB70" s="8" t="inlineStr">
         <is>
@@ -7044,7 +7360,11 @@
       <c r="AU70" s="8" t="n"/>
       <c r="AV70" s="8" t="n"/>
       <c r="AW70" s="8" t="n"/>
-      <c r="AX70" s="8" t="n"/>
+      <c r="AX70" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V3.0 (Generic Assumed)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="n"/>
@@ -7068,12 +7388,12 @@
       </c>
       <c r="H71" s="8" t="inlineStr">
         <is>
-          <t>Terrazzo plaster</t>
+          <t>Terrazzo plastering</t>
         </is>
       </c>
       <c r="I71" s="8" t="inlineStr">
         <is>
-          <t>Cement, Coarse sand, Marble chips, Marble powder</t>
+          <t>Cement, Sand, Marble chips, Marble powder</t>
         </is>
       </c>
       <c r="J71" s="8" t="inlineStr">
@@ -7109,12 +7429,16 @@
       <c r="V71" s="8" t="n"/>
       <c r="W71" s="8" t="n"/>
       <c r="X71" s="8" t="n"/>
-      <c r="Y71" s="8" t="n"/>
-      <c r="Z71" s="8" t="n"/>
+      <c r="Y71" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="Z71" s="17" t="n">
+        <v>0.95</v>
+      </c>
       <c r="AA71" s="8" t="n"/>
       <c r="AB71" s="8" t="inlineStr">
         <is>
-          <t>5.31/13.24.1</t>
+          <t>13.41</t>
         </is>
       </c>
       <c r="AC71" s="8" t="n"/>
@@ -7140,7 +7464,11 @@
       <c r="AU71" s="8" t="n"/>
       <c r="AV71" s="8" t="n"/>
       <c r="AW71" s="8" t="n"/>
-      <c r="AX71" s="8" t="n"/>
+      <c r="AX71" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V3.0 (Generic Assumed)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="8" t="n"/>
@@ -7164,7 +7492,7 @@
       </c>
       <c r="H72" s="8" t="inlineStr">
         <is>
-          <t>Cement mortar</t>
+          <t>Cement mortar plaster</t>
         </is>
       </c>
       <c r="I72" s="8" t="inlineStr">
@@ -7205,12 +7533,16 @@
       <c r="V72" s="8" t="n"/>
       <c r="W72" s="8" t="n"/>
       <c r="X72" s="8" t="n"/>
-      <c r="Y72" s="8" t="n"/>
-      <c r="Z72" s="8" t="n"/>
+      <c r="Y72" s="17" t="n">
+        <v>147.25</v>
+      </c>
+      <c r="Z72" s="17" t="n">
+        <v>0.95</v>
+      </c>
       <c r="AA72" s="8" t="n"/>
       <c r="AB72" s="8" t="inlineStr">
         <is>
-          <t>13.70.1</t>
+          <t>5.31/13.24.1</t>
         </is>
       </c>
       <c r="AC72" s="8" t="n"/>
@@ -7234,7 +7566,11 @@
       <c r="AU72" s="8" t="n"/>
       <c r="AV72" s="8" t="n"/>
       <c r="AW72" s="8" t="n"/>
-      <c r="AX72" s="8" t="n"/>
+      <c r="AX72" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V3.0 (Generic Assumed)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="n"/>
@@ -7258,7 +7594,7 @@
       </c>
       <c r="H73" s="8" t="inlineStr">
         <is>
-          <t>Lime wash</t>
+          <t>Lime white wash</t>
         </is>
       </c>
       <c r="I73" s="8" t="inlineStr">
@@ -7295,12 +7631,16 @@
       <c r="V73" s="8" t="n"/>
       <c r="W73" s="8" t="n"/>
       <c r="X73" s="8" t="n"/>
-      <c r="Y73" s="8" t="n"/>
-      <c r="Z73" s="8" t="n"/>
+      <c r="Y73" s="17" t="n">
+        <v>270.75</v>
+      </c>
+      <c r="Z73" s="17" t="n">
+        <v>0.95</v>
+      </c>
       <c r="AA73" s="8" t="n"/>
       <c r="AB73" s="8" t="inlineStr">
         <is>
-          <t>13.73.1</t>
+          <t>13.70.1</t>
         </is>
       </c>
       <c r="AC73" s="8" t="n"/>
@@ -7324,7 +7664,11 @@
       <c r="AU73" s="8" t="n"/>
       <c r="AV73" s="8" t="n"/>
       <c r="AW73" s="8" t="n"/>
-      <c r="AX73" s="8" t="n"/>
+      <c r="AX73" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V3.0 (Generic Assumed)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="8" t="n"/>
@@ -7337,7 +7681,7 @@
       <c r="D74" s="8" t="n"/>
       <c r="E74" s="8" t="inlineStr">
         <is>
-          <t>Colour washing such as green, blue or buff to give an even shade on new work (two. or more coats) with a base coat of white washing with lime.</t>
+          <t>Colour washing such as green, blue or buff to give an even shade on new work (two or more coats) with a base coat of white washing with lime.</t>
         </is>
       </c>
       <c r="F74" s="8" t="n"/>
@@ -7353,7 +7697,7 @@
       </c>
       <c r="I74" s="8" t="inlineStr">
         <is>
-          <t>Lime</t>
+          <t>Lime, Colour wash</t>
         </is>
       </c>
       <c r="J74" s="8" t="inlineStr">
@@ -7385,12 +7729,16 @@
       <c r="V74" s="8" t="n"/>
       <c r="W74" s="8" t="n"/>
       <c r="X74" s="8" t="n"/>
-      <c r="Y74" s="8" t="n"/>
-      <c r="Z74" s="8" t="n"/>
+      <c r="Y74" s="17" t="n">
+        <v>270.75</v>
+      </c>
+      <c r="Z74" s="17" t="n">
+        <v>0.95</v>
+      </c>
       <c r="AA74" s="8" t="n"/>
       <c r="AB74" s="8" t="inlineStr">
         <is>
-          <t>13.81.1</t>
+          <t>13.73.1</t>
         </is>
       </c>
       <c r="AC74" s="8" t="n"/>
@@ -7414,7 +7762,11 @@
       <c r="AU74" s="8" t="n"/>
       <c r="AV74" s="8" t="n"/>
       <c r="AW74" s="8" t="n"/>
-      <c r="AX74" s="8" t="n"/>
+      <c r="AX74" s="8" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V3.0 (Generic Assumed)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="B75" t="inlineStr">
@@ -7424,7 +7776,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Applying priming coat with ready mixed pink or gray primer of approved brand and manufacture on wood work (hard and soft wood)</t>
+          <t>Applying priming coat with ready mixed pink or gray primer of approved brand and manufacture - on wood work (hard and soft wood)</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -7434,7 +7786,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Primer</t>
+          <t>Wood primer</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -7461,9 +7813,20 @@
       <c r="Q75" s="18" t="n">
         <v>47</v>
       </c>
+      <c r="Y75" s="18" t="n">
+        <v>44.65</v>
+      </c>
+      <c r="Z75" s="18" t="n">
+        <v>0.95</v>
+      </c>
       <c r="AB75" t="inlineStr">
         <is>
-          <t>13.81.4</t>
+          <t>13.81.1</t>
+        </is>
+      </c>
+      <c r="AX75" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V3.0 (Generic Assumed)</t>
         </is>
       </c>
     </row>
@@ -7512,9 +7875,20 @@
       <c r="Q76" s="18" t="n">
         <v>30</v>
       </c>
+      <c r="Y76" s="18" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="Z76" s="18" t="n">
+        <v>0.95</v>
+      </c>
       <c r="AB76" t="inlineStr">
         <is>
-          <t>13.84.3</t>
+          <t>13.81.4</t>
+        </is>
+      </c>
+      <c r="AX76" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V3.0 (Generic Assumed)</t>
         </is>
       </c>
     </row>
@@ -7563,14 +7937,25 @@
       <c r="R77" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="Y77" s="18" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="Z77" s="18" t="n">
+        <v>0.95</v>
+      </c>
       <c r="AB77" t="inlineStr">
         <is>
-          <t>13.94.1</t>
+          <t>13.84.3</t>
         </is>
       </c>
       <c r="AT77" s="18" t="n">
         <v>100</v>
       </c>
+      <c r="AX77" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V3.0 (Generic Assumed)</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="B78" t="inlineStr">
@@ -7617,6 +8002,22 @@
       <c r="Q78" s="18" t="n">
         <v>77</v>
       </c>
+      <c r="Y78" s="18" t="n">
+        <v>73.15000000000001</v>
+      </c>
+      <c r="Z78" s="18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AB78" t="inlineStr">
+        <is>
+          <t>13.94.1</t>
+        </is>
+      </c>
+      <c r="AX78" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V3.0 (Generic Assumed)</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="B79" t="inlineStr">
@@ -7636,12 +8037,12 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>French polish</t>
+          <t>French spirit polish</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>French polish, Wood filler</t>
+          <t>French spirit polish, Wood filler</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -7663,9 +8064,20 @@
       <c r="Q79" s="18" t="n">
         <v>13</v>
       </c>
+      <c r="Y79" s="18" t="n">
+        <v>12.35</v>
+      </c>
+      <c r="Z79" s="18" t="n">
+        <v>0.95</v>
+      </c>
       <c r="AB79" t="inlineStr">
         <is>
           <t>13.101.1</t>
+        </is>
+      </c>
+      <c r="AX79" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V3.0 (Generic Assumed)</t>
         </is>
       </c>
     </row>
@@ -7687,12 +8099,12 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Cement concrete</t>
+          <t>Cement concrete plinth protection</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Cement, Coarse sand, Graded stone aggregate, Brick ballast, Fine sand</t>
+          <t>Cement, Coarse sand, Stone aggregate, Brick ballast, Fine sand</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -7701,7 +8113,7 @@
         </is>
       </c>
       <c r="K80" s="18" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="M80" t="inlineStr">
         <is>
@@ -7719,6 +8131,12 @@
       <c r="Q80" s="18" t="n">
         <v>34.6</v>
       </c>
+      <c r="Y80" s="18" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="Z80" s="18" t="n">
+        <v>0.149</v>
+      </c>
       <c r="AB80" t="inlineStr">
         <is>
           <t>16.1</t>
@@ -7726,6 +8144,11 @@
       </c>
       <c r="AR80" s="18" t="n">
         <v>50</v>
+      </c>
+      <c r="AX80" t="inlineStr">
+        <is>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: added meta data
</commit_message>
<xml_diff>
--- a/output/passport_filled.xlsx
+++ b/output/passport_filled.xlsx
@@ -1748,7 +1748,7 @@
       <c r="AW12" s="8" t="n"/>
       <c r="AX12" s="8" t="inlineStr">
         <is>
-          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M5 inferred from nominal mix 1:5:10 (IS 456); not printed in BoQ</t>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M5 inferred from nominal mix 1:5:10 (IS 456)</t>
         </is>
       </c>
     </row>
@@ -1870,7 +1870,7 @@
       <c r="AW13" s="8" t="n"/>
       <c r="AX13" s="8" t="inlineStr">
         <is>
-          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M5 inferred from nominal mix 1:5:10 (IS 456); not printed in BoQ</t>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M5 inferred from nominal mix 1:5:10 (IS 456)</t>
         </is>
       </c>
     </row>
@@ -1992,7 +1992,7 @@
       <c r="AW14" s="8" t="n"/>
       <c r="AX14" s="8" t="inlineStr">
         <is>
-          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456); not printed in BoQ</t>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2126,7 @@
       <c r="AW15" s="8" t="n"/>
       <c r="AX15" s="8" t="inlineStr">
         <is>
-          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456); not printed in BoQ</t>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2354,7 @@
       <c r="AW17" s="8" t="n"/>
       <c r="AX17" s="8" t="inlineStr">
         <is>
-          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456); not printed in BoQ</t>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
         </is>
       </c>
     </row>
@@ -2476,7 +2476,7 @@
       <c r="AW18" s="8" t="n"/>
       <c r="AX18" s="8" t="inlineStr">
         <is>
-          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456); not printed in BoQ</t>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
         </is>
       </c>
     </row>
@@ -2598,7 +2598,7 @@
       <c r="AW19" s="8" t="n"/>
       <c r="AX19" s="8" t="inlineStr">
         <is>
-          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456); not printed in BoQ</t>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
         </is>
       </c>
     </row>
@@ -2720,7 +2720,7 @@
       <c r="AW20" s="8" t="n"/>
       <c r="AX20" s="8" t="inlineStr">
         <is>
-          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456); not printed in BoQ</t>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
         </is>
       </c>
     </row>
@@ -2842,7 +2842,7 @@
       <c r="AW21" s="8" t="n"/>
       <c r="AX21" s="8" t="inlineStr">
         <is>
-          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456); not printed in BoQ</t>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3722,7 @@
       <c r="AW29" s="8" t="n"/>
       <c r="AX29" s="8" t="inlineStr">
         <is>
-          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456); not printed in BoQ</t>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       <c r="AW54" s="8" t="n"/>
       <c r="AX54" s="8" t="inlineStr">
         <is>
-          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456); not printed in BoQ</t>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
         </is>
       </c>
     </row>
@@ -7526,7 +7526,7 @@
       <c r="AW61" s="8" t="n"/>
       <c r="AX61" s="8" t="inlineStr">
         <is>
-          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M10 inferred from nominal mix 1:3:6 (IS 456); not printed in BoQ</t>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M10 inferred from nominal mix 1:3:6 (IS 456)</t>
         </is>
       </c>
     </row>
@@ -7654,7 +7654,7 @@
       <c r="AW62" s="8" t="n"/>
       <c r="AX62" s="8" t="inlineStr">
         <is>
-          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456); not printed in BoQ</t>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
         </is>
       </c>
     </row>
@@ -9604,7 +9604,7 @@
       </c>
       <c r="AX80" t="inlineStr">
         <is>
-          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M10 inferred from nominal mix 1:3:6 (IS 456); not printed in BoQ</t>
+          <t>EPD Source: ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M10 inferred from nominal mix 1:3:6 (IS 456)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed bug in build file
</commit_message>
<xml_diff>
--- a/output/passport_filled.xlsx
+++ b/output/passport_filled.xlsx
@@ -940,7 +940,7 @@
       </c>
       <c r="H4" s="8" t="inlineStr">
         <is>
-          <t>Soil</t>
+          <t>Earth</t>
         </is>
       </c>
       <c r="I4" s="8" t="inlineStr">
@@ -994,7 +994,7 @@
       <c r="AC4" s="8" t="n"/>
       <c r="AD4" s="8" t="inlineStr">
         <is>
-          <t>Earthwork &gt; Soil</t>
+          <t>Earthwork &gt; Earth</t>
         </is>
       </c>
       <c r="AE4" s="8" t="n"/>
@@ -1015,10 +1015,14 @@
       <c r="AT4" s="8" t="n"/>
       <c r="AU4" s="8" t="n"/>
       <c r="AV4" s="8" t="n"/>
-      <c r="AW4" s="8" t="n"/>
+      <c r="AW4" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX4" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Soil — earthwork/excavated soil; negligible embodied material carbon</t>
+          <t>[EXCLUDED] material: Earth — earthwork/excavated soil; negligible embodied material carbon</t>
         </is>
       </c>
     </row>
@@ -1052,12 +1056,12 @@
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>Earth</t>
+          <t>Excavated earth</t>
         </is>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>Earth</t>
+          <t>Earth, Water</t>
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr">
@@ -1106,7 +1110,7 @@
       <c r="AC5" s="8" t="n"/>
       <c r="AD5" s="8" t="inlineStr">
         <is>
-          <t>Earthwork &gt; Earth</t>
+          <t>Earthwork &gt; Excavated earth</t>
         </is>
       </c>
       <c r="AE5" s="8" t="n"/>
@@ -1129,10 +1133,14 @@
       <c r="AT5" s="8" t="n"/>
       <c r="AU5" s="8" t="n"/>
       <c r="AV5" s="8" t="n"/>
-      <c r="AW5" s="8" t="n"/>
+      <c r="AW5" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX5" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Earth — earthwork/excavated soil; negligible embodied material carbon</t>
+          <t>[EXCLUDED] material: Excavated earth — earthwork/excavated soil; negligible embodied material carbon</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1179,7 @@
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>Sand</t>
+          <t>Sand, Water</t>
         </is>
       </c>
       <c r="J6" s="8" t="inlineStr">
@@ -1241,7 +1249,11 @@
       <c r="AT6" s="8" t="n"/>
       <c r="AU6" s="8" t="n"/>
       <c r="AV6" s="8" t="n"/>
-      <c r="AW6" s="8" t="n"/>
+      <c r="AW6" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX6" s="8" t="inlineStr">
         <is>
           <t>[EXCLUDED] material: Fine sand — earthwork/excavated soil; negligible embodied material carbon</t>
@@ -1299,7 +1311,7 @@
       <c r="L7" s="8" t="n"/>
       <c r="M7" s="8" t="n"/>
       <c r="N7" s="17" t="n">
-        <v>140</v>
+        <v>540</v>
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
@@ -1308,7 +1320,7 @@
       </c>
       <c r="P7" s="8" t="n"/>
       <c r="Q7" s="17" t="n">
-        <v>140</v>
+        <v>540</v>
       </c>
       <c r="R7" s="8" t="n"/>
       <c r="S7" s="8" t="n"/>
@@ -1355,7 +1367,11 @@
       <c r="AT7" s="8" t="n"/>
       <c r="AU7" s="8" t="n"/>
       <c r="AV7" s="8" t="n"/>
-      <c r="AW7" s="8" t="n"/>
+      <c r="AW7" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX7" s="8" t="inlineStr">
         <is>
           <t>[EXCLUDED] material: Soil — earthwork/excavated soil; negligible embodied material carbon</t>
@@ -1397,7 +1413,7 @@
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>Chemical emulsion, Aldrin Emulsifiable Concentrate</t>
+          <t>Aldrin chemical emulsion</t>
         </is>
       </c>
       <c r="J8" s="8" t="inlineStr">
@@ -1467,7 +1483,11 @@
       <c r="AT8" s="8" t="n"/>
       <c r="AU8" s="8" t="n"/>
       <c r="AV8" s="8" t="n"/>
-      <c r="AW8" s="8" t="n"/>
+      <c r="AW8" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX8" s="8" t="inlineStr">
         <is>
           <t>[EXCLUDED] material: Aldrin Emulsifiable Concentrate — category 'Other' not in current EPD database; carbon not estimated</t>
@@ -1593,7 +1613,11 @@
       <c r="AT9" s="8" t="n"/>
       <c r="AU9" s="8" t="n"/>
       <c r="AV9" s="8" t="n"/>
-      <c r="AW9" s="8" t="n"/>
+      <c r="AW9" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX9" s="8" t="inlineStr">
         <is>
           <t>[OK] material: Cement concrete — mass 19200.0 kg [direct volume] × 0.149 kgCO2e/kg = 2860.8 kgCO2e — ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M5 inferred from nominal mix 1:5:10 (IS 456)</t>
@@ -1719,7 +1743,11 @@
       <c r="AT10" s="8" t="n"/>
       <c r="AU10" s="8" t="n"/>
       <c r="AV10" s="8" t="n"/>
-      <c r="AW10" s="8" t="n"/>
+      <c r="AW10" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX10" s="8" t="inlineStr">
         <is>
           <t>[OK] material: Cement concrete — mass 17520.0 kg [direct volume] × 0.149 kgCO2e/kg = 2610.48 kgCO2e — ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M5 inferred from nominal mix 1:5:10 (IS 456)</t>
@@ -1845,7 +1873,11 @@
       <c r="AT11" s="8" t="n"/>
       <c r="AU11" s="8" t="n"/>
       <c r="AV11" s="8" t="n"/>
-      <c r="AW11" s="8" t="n"/>
+      <c r="AW11" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX11" s="8" t="inlineStr">
         <is>
           <t>[OK] material: Cement concrete — mass 240.0 kg [direct volume] × 0.149 kgCO2e/kg = 35.76 kgCO2e — ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
@@ -1983,7 +2015,11 @@
       <c r="AT12" s="8" t="n"/>
       <c r="AU12" s="8" t="n"/>
       <c r="AV12" s="8" t="n"/>
-      <c r="AW12" s="8" t="n"/>
+      <c r="AW12" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX12" s="8" t="inlineStr">
         <is>
           <t>[OK] material: Cement concrete — mass 1382.4 kg [area × thickness (derived)] × 0.149 kgCO2e/kg = 205.98 kgCO2e — ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
@@ -2030,7 +2066,7 @@
       </c>
       <c r="J13" s="8" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Paint/Finish</t>
         </is>
       </c>
       <c r="K13" s="8" t="inlineStr">
@@ -2058,9 +2094,13 @@
       <c r="U13" s="8" t="n"/>
       <c r="V13" s="8" t="n"/>
       <c r="W13" s="8" t="n"/>
-      <c r="X13" s="8" t="n"/>
+      <c r="X13" s="17" t="n">
+        <v>1300</v>
+      </c>
       <c r="Y13" s="8" t="n"/>
-      <c r="Z13" s="8" t="n"/>
+      <c r="Z13" s="17" t="n">
+        <v>0.95</v>
+      </c>
       <c r="AA13" s="8" t="inlineStr">
         <is>
           <t>DSR 1989</t>
@@ -2074,7 +2114,7 @@
       <c r="AC13" s="8" t="n"/>
       <c r="AD13" s="8" t="inlineStr">
         <is>
-          <t>Other &gt; Residual petroleum bitumen</t>
+          <t>Paint/Finish &gt; Residual petroleum bitumen</t>
         </is>
       </c>
       <c r="AE13" s="8" t="n"/>
@@ -2095,10 +2135,14 @@
       <c r="AT13" s="8" t="n"/>
       <c r="AU13" s="8" t="n"/>
       <c r="AV13" s="8" t="n"/>
-      <c r="AW13" s="8" t="n"/>
+      <c r="AW13" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX13" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Residual petroleum bitumen — category 'Other' not in current EPD database; carbon not estimated</t>
+          <t>[EXCLUDED] material: Residual petroleum bitumen — category 'Paint/Finish' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2265,11 @@
       <c r="AT14" s="8" t="n"/>
       <c r="AU14" s="8" t="n"/>
       <c r="AV14" s="8" t="n"/>
-      <c r="AW14" s="8" t="n"/>
+      <c r="AW14" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX14" s="8" t="inlineStr">
         <is>
           <t>[OK] material: Reinforced cement concrete — mass 27120.0 kg [direct volume] × 0.149 kgCO2e/kg = 4040.88 kgCO2e — ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
@@ -2347,7 +2395,11 @@
       <c r="AT15" s="8" t="n"/>
       <c r="AU15" s="8" t="n"/>
       <c r="AV15" s="8" t="n"/>
-      <c r="AW15" s="8" t="n"/>
+      <c r="AW15" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX15" s="8" t="inlineStr">
         <is>
           <t>[OK] material: Reinforced cement concrete — mass 2400.0 kg [direct volume] × 0.149 kgCO2e/kg = 357.6 kgCO2e — ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
@@ -2473,7 +2525,11 @@
       <c r="AT16" s="8" t="n"/>
       <c r="AU16" s="8" t="n"/>
       <c r="AV16" s="8" t="n"/>
-      <c r="AW16" s="8" t="n"/>
+      <c r="AW16" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX16" s="8" t="inlineStr">
         <is>
           <t>[OK] material: Reinforced cement concrete — mass 1440.0 kg [direct volume] × 0.149 kgCO2e/kg = 214.56 kgCO2e — ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
@@ -2495,7 +2551,7 @@
       <c r="D17" s="8" t="n"/>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>Reinforced cement concrete work in lintels, beams, plinth beams and bressummers upto floor two level excluding the cost of centring, shuttering, finishing and reinforcement with 1:2:4 (1 cement : 2 coarse sand : 4 graded stone aggregate 20 mm nominal size).</t>
+          <t>Reinforced cement concrete work in lintels, beams, plinth beams and bresummers upto floor two level excluding the cost of centring, shuttering, finishing and reinforcement with 1:2:4 (1 cement : 2 coarse sand : 4 graded stone aggregate 20 mm nominal size).</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -2599,7 +2655,11 @@
       <c r="AT17" s="8" t="n"/>
       <c r="AU17" s="8" t="n"/>
       <c r="AV17" s="8" t="n"/>
-      <c r="AW17" s="8" t="n"/>
+      <c r="AW17" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX17" s="8" t="inlineStr">
         <is>
           <t>[OK] material: Reinforced cement concrete — mass 4080.0 kg [direct volume] × 0.149 kgCO2e/kg = 607.92 kgCO2e — ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
@@ -2725,7 +2785,11 @@
       <c r="AT18" s="8" t="n"/>
       <c r="AU18" s="8" t="n"/>
       <c r="AV18" s="8" t="n"/>
-      <c r="AW18" s="8" t="n"/>
+      <c r="AW18" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX18" s="8" t="inlineStr">
         <is>
           <t>[OK] material: Reinforced cement concrete — mass 240.0 kg [direct volume] × 0.149 kgCO2e/kg = 35.76 kgCO2e — ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
@@ -2740,14 +2804,14 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>16i</t>
+          <t>16 i</t>
         </is>
       </c>
       <c r="C19" s="8" t="n"/>
       <c r="D19" s="8" t="n"/>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Centring and shuttering including strutting, proping etc. and removal of form work for : i) Suspended floors, roofs, landings balconies and chajjas.</t>
+          <t>Centring and shuttering including strutting, proping etc. and removal of form work for : Suspended floors, roofs, landings balconies and chajjas.</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -2762,17 +2826,17 @@
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>Formwork</t>
+          <t>Formwork shuttering</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>Formwork</t>
+          <t>Timber/Steel formwork</t>
         </is>
       </c>
       <c r="J19" s="8" t="inlineStr">
         <is>
-          <t>Timber</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="K19" s="8" t="inlineStr">
@@ -2800,13 +2864,9 @@
       <c r="U19" s="8" t="n"/>
       <c r="V19" s="8" t="n"/>
       <c r="W19" s="8" t="n"/>
-      <c r="X19" s="17" t="n">
-        <v>750</v>
-      </c>
+      <c r="X19" s="8" t="n"/>
       <c r="Y19" s="8" t="n"/>
-      <c r="Z19" s="17" t="n">
-        <v>0.306</v>
-      </c>
+      <c r="Z19" s="8" t="n"/>
       <c r="AA19" s="8" t="inlineStr">
         <is>
           <t>DSR 1989</t>
@@ -2820,7 +2880,7 @@
       <c r="AC19" s="8" t="n"/>
       <c r="AD19" s="8" t="inlineStr">
         <is>
-          <t>Timber &gt; Formwork</t>
+          <t>Other &gt; Formwork shuttering</t>
         </is>
       </c>
       <c r="AE19" s="8" t="n"/>
@@ -2841,10 +2901,14 @@
       <c r="AT19" s="8" t="n"/>
       <c r="AU19" s="8" t="n"/>
       <c r="AV19" s="8" t="n"/>
-      <c r="AW19" s="8" t="n"/>
+      <c r="AW19" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX19" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Formwork — category 'Timber' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: Formwork shuttering — category 'Other' not in current EPD database; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -2856,14 +2920,14 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>16ii</t>
+          <t>16 ii</t>
         </is>
       </c>
       <c r="C20" s="8" t="n"/>
       <c r="D20" s="8" t="n"/>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>Centring and shuttering including strutting, proping etc. and removal of form work for : ii) Shelves</t>
+          <t>Centring and shuttering including strutting, proping etc. and removal of form work for : Shelves</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -2878,17 +2942,17 @@
       </c>
       <c r="H20" s="8" t="inlineStr">
         <is>
-          <t>Formwork</t>
+          <t>Formwork shuttering</t>
         </is>
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>Formwork</t>
+          <t>Timber/Steel formwork</t>
         </is>
       </c>
       <c r="J20" s="8" t="inlineStr">
         <is>
-          <t>Timber</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="K20" s="8" t="inlineStr">
@@ -2916,13 +2980,9 @@
       <c r="U20" s="8" t="n"/>
       <c r="V20" s="8" t="n"/>
       <c r="W20" s="8" t="n"/>
-      <c r="X20" s="17" t="n">
-        <v>750</v>
-      </c>
+      <c r="X20" s="8" t="n"/>
       <c r="Y20" s="8" t="n"/>
-      <c r="Z20" s="17" t="n">
-        <v>0.306</v>
-      </c>
+      <c r="Z20" s="8" t="n"/>
       <c r="AA20" s="8" t="inlineStr">
         <is>
           <t>DSR 1989</t>
@@ -2936,7 +2996,7 @@
       <c r="AC20" s="8" t="n"/>
       <c r="AD20" s="8" t="inlineStr">
         <is>
-          <t>Timber &gt; Formwork</t>
+          <t>Other &gt; Formwork shuttering</t>
         </is>
       </c>
       <c r="AE20" s="8" t="n"/>
@@ -2957,10 +3017,14 @@
       <c r="AT20" s="8" t="n"/>
       <c r="AU20" s="8" t="n"/>
       <c r="AV20" s="8" t="n"/>
-      <c r="AW20" s="8" t="n"/>
+      <c r="AW20" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX20" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Formwork — category 'Timber' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: Formwork shuttering — category 'Other' not in current EPD database; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -2972,14 +3036,14 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>16iii</t>
+          <t>16 iii</t>
         </is>
       </c>
       <c r="C21" s="8" t="n"/>
       <c r="D21" s="8" t="n"/>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Centring and shuttering including strutting, proping etc. and removal of form work for : iii) Lintels, beams, plinth beams, girders bressumers and cantilever.</t>
+          <t>Centring and shuttering including strutting, proping etc. and removal of form work for : Lintels, beams, plinth beams, girders bressumers and cantilever.</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -2994,17 +3058,17 @@
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>Formwork</t>
+          <t>Formwork shuttering</t>
         </is>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>Formwork</t>
+          <t>Timber/Steel formwork</t>
         </is>
       </c>
       <c r="J21" s="8" t="inlineStr">
         <is>
-          <t>Timber</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="K21" s="8" t="inlineStr">
@@ -3032,13 +3096,9 @@
       <c r="U21" s="8" t="n"/>
       <c r="V21" s="8" t="n"/>
       <c r="W21" s="8" t="n"/>
-      <c r="X21" s="17" t="n">
-        <v>750</v>
-      </c>
+      <c r="X21" s="8" t="n"/>
       <c r="Y21" s="8" t="n"/>
-      <c r="Z21" s="17" t="n">
-        <v>0.306</v>
-      </c>
+      <c r="Z21" s="8" t="n"/>
       <c r="AA21" s="8" t="inlineStr">
         <is>
           <t>DSR 1989</t>
@@ -3052,7 +3112,7 @@
       <c r="AC21" s="8" t="n"/>
       <c r="AD21" s="8" t="inlineStr">
         <is>
-          <t>Timber &gt; Formwork</t>
+          <t>Other &gt; Formwork shuttering</t>
         </is>
       </c>
       <c r="AE21" s="8" t="n"/>
@@ -3073,10 +3133,14 @@
       <c r="AT21" s="8" t="n"/>
       <c r="AU21" s="8" t="n"/>
       <c r="AV21" s="8" t="n"/>
-      <c r="AW21" s="8" t="n"/>
+      <c r="AW21" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX21" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Formwork — category 'Timber' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: Formwork shuttering — category 'Other' not in current EPD database; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -3088,14 +3152,14 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>16iv</t>
+          <t>16 iv</t>
         </is>
       </c>
       <c r="C22" s="8" t="n"/>
       <c r="D22" s="8" t="n"/>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>Centring and shuttering including strutting, proping etc. and removal of form work for : iv) Columns, pillars, posts and struts.</t>
+          <t>Centring and shuttering including strutting, proping etc. and removal of form work for : Columns, pillars, posts and struts.</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -3110,17 +3174,17 @@
       </c>
       <c r="H22" s="8" t="inlineStr">
         <is>
-          <t>Formwork</t>
+          <t>Formwork shuttering</t>
         </is>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
-          <t>Formwork</t>
+          <t>Timber/Steel formwork</t>
         </is>
       </c>
       <c r="J22" s="8" t="inlineStr">
         <is>
-          <t>Timber</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="K22" s="8" t="inlineStr">
@@ -3148,13 +3212,9 @@
       <c r="U22" s="8" t="n"/>
       <c r="V22" s="8" t="n"/>
       <c r="W22" s="8" t="n"/>
-      <c r="X22" s="17" t="n">
-        <v>750</v>
-      </c>
+      <c r="X22" s="8" t="n"/>
       <c r="Y22" s="8" t="n"/>
-      <c r="Z22" s="17" t="n">
-        <v>0.306</v>
-      </c>
+      <c r="Z22" s="8" t="n"/>
       <c r="AA22" s="8" t="inlineStr">
         <is>
           <t>DSR 1989</t>
@@ -3168,7 +3228,7 @@
       <c r="AC22" s="8" t="n"/>
       <c r="AD22" s="8" t="inlineStr">
         <is>
-          <t>Timber &gt; Formwork</t>
+          <t>Other &gt; Formwork shuttering</t>
         </is>
       </c>
       <c r="AE22" s="8" t="n"/>
@@ -3189,10 +3249,14 @@
       <c r="AT22" s="8" t="n"/>
       <c r="AU22" s="8" t="n"/>
       <c r="AV22" s="8" t="n"/>
-      <c r="AW22" s="8" t="n"/>
+      <c r="AW22" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX22" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Formwork — category 'Timber' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: Formwork shuttering — category 'Other' not in current EPD database; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -3204,14 +3268,14 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>16v</t>
+          <t>16 v</t>
         </is>
       </c>
       <c r="C23" s="8" t="n"/>
       <c r="D23" s="8" t="n"/>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>Centring and shuttering including strutting, proping etc. and removal of form work for : v) Vertical and horizontal fins individually or forming box louvers hand and facias.</t>
+          <t>Centring and shuttering including strutting, proping etc. and removal of form work for : Vertical and horizontal fins individually or forming box louvers hand and facias.</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -3226,17 +3290,17 @@
       </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
-          <t>Formwork</t>
+          <t>Formwork shuttering</t>
         </is>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
-          <t>Formwork</t>
+          <t>Timber/Steel formwork</t>
         </is>
       </c>
       <c r="J23" s="8" t="inlineStr">
         <is>
-          <t>Timber</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="K23" s="8" t="inlineStr">
@@ -3264,13 +3328,9 @@
       <c r="U23" s="8" t="n"/>
       <c r="V23" s="8" t="n"/>
       <c r="W23" s="8" t="n"/>
-      <c r="X23" s="17" t="n">
-        <v>750</v>
-      </c>
+      <c r="X23" s="8" t="n"/>
       <c r="Y23" s="8" t="n"/>
-      <c r="Z23" s="17" t="n">
-        <v>0.306</v>
-      </c>
+      <c r="Z23" s="8" t="n"/>
       <c r="AA23" s="8" t="inlineStr">
         <is>
           <t>DSR 1989</t>
@@ -3284,7 +3344,7 @@
       <c r="AC23" s="8" t="n"/>
       <c r="AD23" s="8" t="inlineStr">
         <is>
-          <t>Timber &gt; Formwork</t>
+          <t>Other &gt; Formwork shuttering</t>
         </is>
       </c>
       <c r="AE23" s="8" t="n"/>
@@ -3305,10 +3365,14 @@
       <c r="AT23" s="8" t="n"/>
       <c r="AU23" s="8" t="n"/>
       <c r="AV23" s="8" t="n"/>
-      <c r="AW23" s="8" t="n"/>
+      <c r="AW23" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX23" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Formwork — category 'Timber' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: Formwork shuttering — category 'Other' not in current EPD database; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -3320,14 +3384,14 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>17i</t>
+          <t>17 i</t>
         </is>
       </c>
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="8" t="n"/>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>Reinforcement for RCC work including bending binding and placing in position complete. i) Mild steel and medium tensile steel bars.</t>
+          <t>Reinforcement for RCC work including bending binding and placing in position complete. Mild steel and medium tensile steel bars.</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -3423,7 +3487,11 @@
       <c r="AT24" s="8" t="n"/>
       <c r="AU24" s="8" t="n"/>
       <c r="AV24" s="8" t="n"/>
-      <c r="AW24" s="8" t="n"/>
+      <c r="AW24" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX24" s="8" t="inlineStr">
         <is>
           <t>[OK] material: Mild steel bars — mass 100.0 kg [direct weight] × 1.55 kgCO2e/kg = 155.0 kgCO2e — ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
@@ -3438,14 +3506,14 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>17ii</t>
+          <t>17 ii</t>
         </is>
       </c>
       <c r="C25" s="8" t="n"/>
       <c r="D25" s="8" t="n"/>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>Reinforcement for RCC work including bending binding and placing in position complete. ii) Cold twisted bars</t>
+          <t>Reinforcement for RCC work including bending binding and placing in position complete. Cold twisted bars</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
@@ -3460,12 +3528,12 @@
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>Cold twisted bars</t>
+          <t>Cold twisted steel bars</t>
         </is>
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>Cold twisted steel</t>
         </is>
       </c>
       <c r="J25" s="8" t="inlineStr">
@@ -3520,7 +3588,7 @@
       <c r="AC25" s="8" t="n"/>
       <c r="AD25" s="8" t="inlineStr">
         <is>
-          <t>Steel &gt; Cold twisted bars</t>
+          <t>Steel &gt; Cold twisted steel bars</t>
         </is>
       </c>
       <c r="AE25" s="8" t="n"/>
@@ -3541,10 +3609,14 @@
       <c r="AT25" s="8" t="n"/>
       <c r="AU25" s="8" t="n"/>
       <c r="AV25" s="8" t="n"/>
-      <c r="AW25" s="8" t="n"/>
+      <c r="AW25" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX25" s="8" t="inlineStr">
         <is>
-          <t>[OK] material: Cold twisted bars — mass 1375.0 kg [direct weight] × 1.55 kgCO2e/kg = 2131.25 kgCO2e — ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
+          <t>[OK] material: Cold twisted steel bars — mass 1375.0 kg [direct weight] × 1.55 kgCO2e/kg = 2131.25 kgCO2e — ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
         </is>
       </c>
     </row>
@@ -3667,7 +3739,11 @@
       <c r="AT26" s="8" t="n"/>
       <c r="AU26" s="8" t="n"/>
       <c r="AV26" s="8" t="n"/>
-      <c r="AW26" s="8" t="n"/>
+      <c r="AW26" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX26" s="8" t="inlineStr">
         <is>
           <t>[OK] material: Reinforced cement concrete — mass 1920.0 kg [direct volume] × 0.149 kgCO2e/kg = 286.08 kgCO2e — ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
@@ -3699,12 +3775,12 @@
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>Civil &amp; Sitework</t>
+          <t>Structural</t>
         </is>
       </c>
       <c r="H27" s="8" t="inlineStr">
         <is>
-          <t>Bricks</t>
+          <t>Brick masonry</t>
         </is>
       </c>
       <c r="I27" s="8" t="inlineStr">
@@ -3768,7 +3844,7 @@
       <c r="AC27" s="8" t="n"/>
       <c r="AD27" s="8" t="inlineStr">
         <is>
-          <t>Masonry &gt; Bricks &gt; 1:6</t>
+          <t>Masonry &gt; Brick masonry &gt; 1:6</t>
         </is>
       </c>
       <c r="AE27" s="8" t="n"/>
@@ -3789,10 +3865,14 @@
       <c r="AT27" s="8" t="n"/>
       <c r="AU27" s="8" t="n"/>
       <c r="AV27" s="8" t="n"/>
-      <c r="AW27" s="8" t="n"/>
+      <c r="AW27" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX27" s="8" t="inlineStr">
         <is>
-          <t>[OK] material: Bricks — mass 30600.0 kg [direct volume] × 0.213 kgCO2e/kg = 6517.8 kgCO2e — ICE Database V4.0 (Brick Clay) via NZBG Guide V1.0</t>
+          <t>[OK] material: Brick masonry — mass 30600.0 kg [direct volume] × 0.213 kgCO2e/kg = 6517.8 kgCO2e — ICE Database V4.0 (Brick Clay) via NZBG Guide V1.0</t>
         </is>
       </c>
     </row>
@@ -3821,12 +3901,12 @@
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>Civil &amp; Sitework</t>
+          <t>Structural</t>
         </is>
       </c>
       <c r="H28" s="8" t="inlineStr">
         <is>
-          <t>Bricks</t>
+          <t>Brick masonry</t>
         </is>
       </c>
       <c r="I28" s="8" t="inlineStr">
@@ -3890,7 +3970,7 @@
       <c r="AC28" s="8" t="n"/>
       <c r="AD28" s="8" t="inlineStr">
         <is>
-          <t>Masonry &gt; Bricks &gt; 1:6</t>
+          <t>Masonry &gt; Brick masonry &gt; 1:6</t>
         </is>
       </c>
       <c r="AE28" s="8" t="n"/>
@@ -3911,10 +3991,14 @@
       <c r="AT28" s="8" t="n"/>
       <c r="AU28" s="8" t="n"/>
       <c r="AV28" s="8" t="n"/>
-      <c r="AW28" s="8" t="n"/>
+      <c r="AW28" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX28" s="8" t="inlineStr">
         <is>
-          <t>[OK] material: Bricks — mass 72540.0 kg [direct volume] × 0.213 kgCO2e/kg = 15451.02 kgCO2e — ICE Database V4.0 (Brick Clay) via NZBG Guide V1.0</t>
+          <t>[OK] material: Brick masonry — mass 72540.0 kg [direct volume] × 0.213 kgCO2e/kg = 15451.02 kgCO2e — ICE Database V4.0 (Brick Clay) via NZBG Guide V1.0</t>
         </is>
       </c>
     </row>
@@ -3933,7 +4017,7 @@
       <c r="D29" s="8" t="n"/>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>Brick work 7 cm thick with bricks of class designation ______ in super structure upto floor two level in cement mortar 1:3 (1 cement : 3 coarse sand).</t>
+          <t>Brick work 7 cm thick with bricks of class designation ------ in super structure upto floor two level in cement mortar 1:3 (1 cement : 3 coarse sand).</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
@@ -3943,12 +4027,12 @@
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>Civil &amp; Sitework</t>
+          <t>Structural</t>
         </is>
       </c>
       <c r="H29" s="8" t="inlineStr">
         <is>
-          <t>Bricks</t>
+          <t>Brick masonry</t>
         </is>
       </c>
       <c r="I29" s="8" t="inlineStr">
@@ -4022,7 +4106,7 @@
       <c r="AC29" s="8" t="n"/>
       <c r="AD29" s="8" t="inlineStr">
         <is>
-          <t>Masonry &gt; Bricks &gt; 1:3</t>
+          <t>Masonry &gt; Brick masonry &gt; 1:3</t>
         </is>
       </c>
       <c r="AE29" s="8" t="n"/>
@@ -4045,10 +4129,14 @@
       <c r="AT29" s="8" t="n"/>
       <c r="AU29" s="8" t="n"/>
       <c r="AV29" s="8" t="n"/>
-      <c r="AW29" s="8" t="n"/>
+      <c r="AW29" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX29" s="8" t="inlineStr">
         <is>
-          <t>[OK] material: Bricks — mass 113.4 kg [area × thickness (derived)] × 0.213 kgCO2e/kg = 24.15 kgCO2e — ICE Database V4.0 (Brick Clay) via NZBG Guide V1.0</t>
+          <t>[OK] material: Brick masonry — mass 113.4 kg [area × thickness (derived)] × 0.213 kgCO2e/kg = 24.15 kgCO2e — ICE Database V4.0 (Brick Clay) via NZBG Guide V1.0</t>
         </is>
       </c>
     </row>
@@ -4067,7 +4155,7 @@
       <c r="D30" s="8" t="n"/>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>Half brick masonry with bricks of class designation ______ in foundation &amp; plinth in cement mortar 1:4 (1 cement : 4 coarse sand)</t>
+          <t>Half brick masonry with bricks of class designation _____ in foundation &amp; plinth in cement mortar 1:4 (1 cement : 4 coarse sand)</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
@@ -4077,12 +4165,12 @@
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>Civil &amp; Sitework</t>
+          <t>Structural</t>
         </is>
       </c>
       <c r="H30" s="8" t="inlineStr">
         <is>
-          <t>Bricks</t>
+          <t>Half brick masonry</t>
         </is>
       </c>
       <c r="I30" s="8" t="inlineStr">
@@ -4144,7 +4232,7 @@
       <c r="AC30" s="8" t="n"/>
       <c r="AD30" s="8" t="inlineStr">
         <is>
-          <t>Masonry &gt; Bricks &gt; 1:4</t>
+          <t>Masonry &gt; Half brick masonry &gt; 1:4</t>
         </is>
       </c>
       <c r="AE30" s="8" t="n"/>
@@ -4165,10 +4253,14 @@
       <c r="AT30" s="8" t="n"/>
       <c r="AU30" s="8" t="n"/>
       <c r="AV30" s="8" t="n"/>
-      <c r="AW30" s="8" t="n"/>
+      <c r="AW30" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX30" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Bricks — category 'Masonry' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: Half brick masonry — category 'Masonry' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -4187,7 +4279,7 @@
       <c r="D31" s="8" t="n"/>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>Half brick masonry with bricks of class designation ____ in super structure upto floor two level in cement mortar 1:4 (1 cement : 4 coarse sand).</t>
+          <t>Half brick masonry with bricks of class designation ______ in super structure upto floor two level in cement mortar 1:4 (1 cement : 4 coarse sand).</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
@@ -4197,12 +4289,12 @@
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>Civil &amp; Sitework</t>
+          <t>Structural</t>
         </is>
       </c>
       <c r="H31" s="8" t="inlineStr">
         <is>
-          <t>Bricks</t>
+          <t>Half brick masonry</t>
         </is>
       </c>
       <c r="I31" s="8" t="inlineStr">
@@ -4264,7 +4356,7 @@
       <c r="AC31" s="8" t="n"/>
       <c r="AD31" s="8" t="inlineStr">
         <is>
-          <t>Masonry &gt; Bricks &gt; 1:4</t>
+          <t>Masonry &gt; Half brick masonry &gt; 1:4</t>
         </is>
       </c>
       <c r="AE31" s="8" t="n"/>
@@ -4285,10 +4377,14 @@
       <c r="AT31" s="8" t="n"/>
       <c r="AU31" s="8" t="n"/>
       <c r="AV31" s="8" t="n"/>
-      <c r="AW31" s="8" t="n"/>
+      <c r="AW31" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX31" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Bricks — category 'Masonry' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: Half brick masonry — category 'Masonry' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -4322,7 +4418,7 @@
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>Wood</t>
+          <t>Wood work frame</t>
         </is>
       </c>
       <c r="I32" s="8" t="inlineStr">
@@ -4378,7 +4474,7 @@
       <c r="AC32" s="8" t="n"/>
       <c r="AD32" s="8" t="inlineStr">
         <is>
-          <t>Timber &gt; Wood</t>
+          <t>Timber &gt; Wood work frame</t>
         </is>
       </c>
       <c r="AE32" s="8" t="n"/>
@@ -4399,10 +4495,14 @@
       <c r="AT32" s="8" t="n"/>
       <c r="AU32" s="8" t="n"/>
       <c r="AV32" s="8" t="n"/>
-      <c r="AW32" s="8" t="n"/>
+      <c r="AW32" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX32" s="8" t="inlineStr">
         <is>
-          <t>[OK] material: Wood — mass 26.25 kg [direct volume] × 0.306 kgCO2e/kg = 8.03 kgCO2e — ICE Database V4.0 (Timber Hardwood) via NZBG Guide V1.0</t>
+          <t>[OK] material: Wood work frame — mass 26.25 kg [direct volume] × 0.306 kgCO2e/kg = 8.03 kgCO2e — ICE Database V4.0 (Timber Hardwood) via NZBG Guide V1.0</t>
         </is>
       </c>
     </row>
@@ -4436,12 +4536,12 @@
       </c>
       <c r="H33" s="8" t="inlineStr">
         <is>
-          <t>Wood</t>
+          <t>Wood door shutters</t>
         </is>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
-          <t>Wood, MS</t>
+          <t>Wood, MS butt hinges, Screws</t>
         </is>
       </c>
       <c r="J33" s="8" t="inlineStr">
@@ -4506,7 +4606,7 @@
       <c r="AC33" s="8" t="n"/>
       <c r="AD33" s="8" t="inlineStr">
         <is>
-          <t>Timber &gt; Wood</t>
+          <t>Timber &gt; Wood door shutters</t>
         </is>
       </c>
       <c r="AE33" s="8" t="n"/>
@@ -4529,10 +4629,14 @@
       <c r="AT33" s="8" t="n"/>
       <c r="AU33" s="8" t="n"/>
       <c r="AV33" s="8" t="n"/>
-      <c r="AW33" s="8" t="n"/>
+      <c r="AW33" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX33" s="8" t="inlineStr">
         <is>
-          <t>[OK] material: Wood — mass 472.5 kg [area × thickness (derived)] × 0.306 kgCO2e/kg = 144.59 kgCO2e — ICE Database V4.0 (Timber Hardwood) via NZBG Guide V1.0</t>
+          <t>[OK] material: Wood door shutters — mass 472.5 kg [area × thickness (derived)] × 0.306 kgCO2e/kg = 144.59 kgCO2e — ICE Database V4.0 (Timber Hardwood) via NZBG Guide V1.0</t>
         </is>
       </c>
     </row>
@@ -4566,12 +4670,12 @@
       </c>
       <c r="H34" s="8" t="inlineStr">
         <is>
-          <t>Teak ply veneer</t>
+          <t>Flush door shutters</t>
         </is>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
-          <t>Hard wood, Teak ply, Commercial ply, MS</t>
+          <t>Block board, Hardwood, Teak ply, Commercial ply, Nickel plated MS piano hinges</t>
         </is>
       </c>
       <c r="J34" s="8" t="inlineStr">
@@ -4628,11 +4732,15 @@
           <t>DSR 1989</t>
         </is>
       </c>
-      <c r="AB34" s="8" t="n"/>
+      <c r="AB34" s="8" t="inlineStr">
+        <is>
+          <t>9.51</t>
+        </is>
+      </c>
       <c r="AC34" s="8" t="n"/>
       <c r="AD34" s="8" t="inlineStr">
         <is>
-          <t>Timber &gt; Teak ply veneer</t>
+          <t>Timber &gt; Flush door shutters</t>
         </is>
       </c>
       <c r="AE34" s="8" t="n"/>
@@ -4655,10 +4763,14 @@
       <c r="AT34" s="8" t="n"/>
       <c r="AU34" s="8" t="n"/>
       <c r="AV34" s="8" t="n"/>
-      <c r="AW34" s="8" t="n"/>
+      <c r="AW34" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX34" s="8" t="inlineStr">
         <is>
-          <t>[OK] material: Teak ply veneer — mass 88.12 kg [area × thickness (derived)] × 0.306 kgCO2e/kg = 26.97 kgCO2e — ICE Database V4.0 (Timber Hardwood) via NZBG Guide V1.0</t>
+          <t>[OK] material: Flush door shutters — mass 88.12 kg [area × thickness (derived)] × 0.306 kgCO2e/kg = 26.97 kgCO2e — ICE Database V4.0 (Timber Hardwood) via NZBG Guide V1.0</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4804,7 @@
       </c>
       <c r="H35" s="8" t="inlineStr">
         <is>
-          <t>Teak wood</t>
+          <t>Teak wood plugs</t>
         </is>
       </c>
       <c r="I35" s="8" t="inlineStr">
@@ -4746,15 +4858,11 @@
           <t>DSR 1989</t>
         </is>
       </c>
-      <c r="AB35" s="8" t="inlineStr">
-        <is>
-          <t>9.51</t>
-        </is>
-      </c>
+      <c r="AB35" s="8" t="n"/>
       <c r="AC35" s="8" t="n"/>
       <c r="AD35" s="8" t="inlineStr">
         <is>
-          <t>Timber &gt; Teak wood &gt; 1:3</t>
+          <t>Timber &gt; Teak wood plugs &gt; 1:3</t>
         </is>
       </c>
       <c r="AE35" s="8" t="n"/>
@@ -4776,15 +4884,21 @@
       <c r="AQ35" s="17" t="n">
         <v>50</v>
       </c>
-      <c r="AR35" s="8" t="n"/>
+      <c r="AR35" s="17" t="n">
+        <v>50</v>
+      </c>
       <c r="AS35" s="8" t="n"/>
       <c r="AT35" s="8" t="n"/>
       <c r="AU35" s="8" t="n"/>
       <c r="AV35" s="8" t="n"/>
-      <c r="AW35" s="8" t="n"/>
+      <c r="AW35" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX35" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Teak wood — category 'Timber' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: Teak wood plugs — category 'Timber' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -4803,7 +4917,7 @@
       <c r="D36" s="8" t="n"/>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t>Providing and fixing M.S.oxidised fan light vantilator catch with necessary screws etc. complete.</t>
+          <t>Providing and fixing M.S.oxidised fan light ventilator catch with necessary screws etc. complete.</t>
         </is>
       </c>
       <c r="F36" s="8" t="inlineStr">
@@ -4818,12 +4932,12 @@
       </c>
       <c r="H36" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>M.S. oxidised ventilator catch</t>
         </is>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>M.S., Screws</t>
         </is>
       </c>
       <c r="J36" s="8" t="inlineStr">
@@ -4868,11 +4982,15 @@
           <t>DSR 1989</t>
         </is>
       </c>
-      <c r="AB36" s="8" t="n"/>
+      <c r="AB36" s="8" t="inlineStr">
+        <is>
+          <t>9.127.3</t>
+        </is>
+      </c>
       <c r="AC36" s="8" t="n"/>
       <c r="AD36" s="8" t="inlineStr">
         <is>
-          <t>Steel &gt; Mild steel</t>
+          <t>Steel &gt; M.S. oxidised ventilator catch</t>
         </is>
       </c>
       <c r="AE36" s="8" t="n"/>
@@ -4893,10 +5011,14 @@
       <c r="AT36" s="8" t="n"/>
       <c r="AU36" s="8" t="n"/>
       <c r="AV36" s="8" t="n"/>
-      <c r="AW36" s="8" t="n"/>
+      <c r="AW36" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX36" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Mild steel — category 'Steel' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: M.S. oxidised ventilator catch — category 'Steel' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -4930,12 +5052,12 @@
       </c>
       <c r="H37" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>M.S. hasp and staple</t>
         </is>
       </c>
       <c r="I37" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>Oxidised M.S., Screws</t>
         </is>
       </c>
       <c r="J37" s="8" t="inlineStr">
@@ -4982,13 +5104,13 @@
       </c>
       <c r="AB37" s="8" t="inlineStr">
         <is>
-          <t>9.127.3</t>
+          <t>9.218.1</t>
         </is>
       </c>
       <c r="AC37" s="8" t="n"/>
       <c r="AD37" s="8" t="inlineStr">
         <is>
-          <t>Steel &gt; Mild steel</t>
+          <t>Steel &gt; M.S. hasp and staple</t>
         </is>
       </c>
       <c r="AE37" s="8" t="n"/>
@@ -5011,10 +5133,14 @@
       <c r="AT37" s="8" t="n"/>
       <c r="AU37" s="8" t="n"/>
       <c r="AV37" s="8" t="n"/>
-      <c r="AW37" s="8" t="n"/>
+      <c r="AW37" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX37" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Mild steel — category 'Steel' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: M.S. hasp and staple — category 'Steel' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -5048,12 +5174,12 @@
       </c>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium sliding door bolts</t>
         </is>
       </c>
       <c r="I38" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium, Nuts, Screws</t>
         </is>
       </c>
       <c r="J38" s="8" t="inlineStr">
@@ -5094,15 +5220,11 @@
           <t>DSR 1989</t>
         </is>
       </c>
-      <c r="AB38" s="8" t="inlineStr">
-        <is>
-          <t>9.218.1</t>
-        </is>
-      </c>
+      <c r="AB38" s="8" t="n"/>
       <c r="AC38" s="8" t="n"/>
       <c r="AD38" s="8" t="inlineStr">
         <is>
-          <t>Other &gt; Aluminium</t>
+          <t>Other &gt; Aluminium sliding door bolts</t>
         </is>
       </c>
       <c r="AE38" s="8" t="n"/>
@@ -5127,10 +5249,14 @@
       </c>
       <c r="AU38" s="8" t="n"/>
       <c r="AV38" s="8" t="n"/>
-      <c r="AW38" s="8" t="n"/>
+      <c r="AW38" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX38" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Aluminium — category 'Other' not in current EPD database; carbon not estimated</t>
+          <t>[EXCLUDED] material: Aluminium sliding door bolts — category 'Other' not in current EPD database; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -5142,14 +5268,14 @@
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>31i</t>
+          <t>31 i</t>
         </is>
       </c>
       <c r="C39" s="8" t="n"/>
       <c r="D39" s="8" t="n"/>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>Providing and fixing aluminium tower bolts anodised transparent or dyed to required colour or shade with necessary screws etc. complete. i) 200 x 10 mm</t>
+          <t>Providing and fixing aluminium tower bolts anodised transparent or dyed to required colour or shade with necessary screws etc. complete. 200 x 10 mm</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
@@ -5164,12 +5290,12 @@
       </c>
       <c r="H39" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium tower bolts</t>
         </is>
       </c>
       <c r="I39" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium, Screws</t>
         </is>
       </c>
       <c r="J39" s="8" t="inlineStr">
@@ -5218,7 +5344,7 @@
       <c r="AC39" s="8" t="n"/>
       <c r="AD39" s="8" t="inlineStr">
         <is>
-          <t>Other &gt; Aluminium</t>
+          <t>Other &gt; Aluminium tower bolts</t>
         </is>
       </c>
       <c r="AE39" s="8" t="n"/>
@@ -5243,10 +5369,14 @@
       </c>
       <c r="AU39" s="8" t="n"/>
       <c r="AV39" s="8" t="n"/>
-      <c r="AW39" s="8" t="n"/>
+      <c r="AW39" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX39" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Aluminium — category 'Other' not in current EPD database; carbon not estimated</t>
+          <t>[EXCLUDED] material: Aluminium tower bolts — category 'Other' not in current EPD database; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -5258,14 +5388,14 @@
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>31ii</t>
+          <t>31 ii</t>
         </is>
       </c>
       <c r="C40" s="8" t="n"/>
       <c r="D40" s="8" t="n"/>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t>Providing and fixing aluminium tower bolts anodised transparent or dyed to required colour or shade with necessary screws etc. complete. ii) 100 x 10 mm</t>
+          <t>Providing and fixing aluminium tower bolts anodised transparent or dyed to required colour or shade with necessary screws etc. complete. 100 x 10 mm</t>
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr">
@@ -5280,12 +5410,12 @@
       </c>
       <c r="H40" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium tower bolts</t>
         </is>
       </c>
       <c r="I40" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium, Screws</t>
         </is>
       </c>
       <c r="J40" s="8" t="inlineStr">
@@ -5334,7 +5464,7 @@
       <c r="AC40" s="8" t="n"/>
       <c r="AD40" s="8" t="inlineStr">
         <is>
-          <t>Other &gt; Aluminium</t>
+          <t>Other &gt; Aluminium tower bolts</t>
         </is>
       </c>
       <c r="AE40" s="8" t="n"/>
@@ -5359,10 +5489,14 @@
       </c>
       <c r="AU40" s="8" t="n"/>
       <c r="AV40" s="8" t="n"/>
-      <c r="AW40" s="8" t="n"/>
+      <c r="AW40" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX40" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Aluminium — category 'Other' not in current EPD database; carbon not estimated</t>
+          <t>[EXCLUDED] material: Aluminium tower bolts — category 'Other' not in current EPD database; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -5374,14 +5508,14 @@
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>32i</t>
+          <t>32 i</t>
         </is>
       </c>
       <c r="C41" s="8" t="n"/>
       <c r="D41" s="8" t="n"/>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>Providing and fixing aluminium handles anodised transparent or dyed to required colour or shade with necessary screws etc. complete. i) 100 mm</t>
+          <t>Providing and fixing aluminium handles anodised transparent or dyed to required colour or shade with necessary screws etc. complete. 100 mm</t>
         </is>
       </c>
       <c r="F41" s="8" t="inlineStr">
@@ -5396,12 +5530,12 @@
       </c>
       <c r="H41" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium handles</t>
         </is>
       </c>
       <c r="I41" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium, Screws</t>
         </is>
       </c>
       <c r="J41" s="8" t="inlineStr">
@@ -5450,7 +5584,7 @@
       <c r="AC41" s="8" t="n"/>
       <c r="AD41" s="8" t="inlineStr">
         <is>
-          <t>Other &gt; Aluminium</t>
+          <t>Other &gt; Aluminium handles</t>
         </is>
       </c>
       <c r="AE41" s="8" t="n"/>
@@ -5473,10 +5607,14 @@
       <c r="AT41" s="8" t="n"/>
       <c r="AU41" s="8" t="n"/>
       <c r="AV41" s="8" t="n"/>
-      <c r="AW41" s="8" t="n"/>
+      <c r="AW41" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX41" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Aluminium — category 'Other' not in current EPD database; carbon not estimated</t>
+          <t>[EXCLUDED] material: Aluminium handles — category 'Other' not in current EPD database; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -5488,14 +5626,14 @@
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>32ii</t>
+          <t>32 ii</t>
         </is>
       </c>
       <c r="C42" s="8" t="n"/>
       <c r="D42" s="8" t="n"/>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>Providing and fixing aluminium handles anodised transparent or dyed to required colour or shade with necessary screws etc. complete. ii) 75 mm</t>
+          <t>Providing and fixing aluminium handles anodised transparent or dyed to required colour or shade with necessary screws etc. complete. 75 mm</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
@@ -5510,12 +5648,12 @@
       </c>
       <c r="H42" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium handles</t>
         </is>
       </c>
       <c r="I42" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium, Screws</t>
         </is>
       </c>
       <c r="J42" s="8" t="inlineStr">
@@ -5564,7 +5702,7 @@
       <c r="AC42" s="8" t="n"/>
       <c r="AD42" s="8" t="inlineStr">
         <is>
-          <t>Other &gt; Aluminium</t>
+          <t>Other &gt; Aluminium handles</t>
         </is>
       </c>
       <c r="AE42" s="8" t="n"/>
@@ -5587,10 +5725,14 @@
       <c r="AT42" s="8" t="n"/>
       <c r="AU42" s="8" t="n"/>
       <c r="AV42" s="8" t="n"/>
-      <c r="AW42" s="8" t="n"/>
+      <c r="AW42" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX42" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Aluminium — category 'Other' not in current EPD database; carbon not estimated</t>
+          <t>[EXCLUDED] material: Aluminium handles — category 'Other' not in current EPD database; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -5624,12 +5766,12 @@
       </c>
       <c r="H43" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium hanging floor door stopper</t>
         </is>
       </c>
       <c r="I43" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium, Screws</t>
         </is>
       </c>
       <c r="J43" s="8" t="inlineStr">
@@ -5678,7 +5820,7 @@
       <c r="AC43" s="8" t="n"/>
       <c r="AD43" s="8" t="inlineStr">
         <is>
-          <t>Other &gt; Aluminium</t>
+          <t>Other &gt; Aluminium hanging floor door stopper</t>
         </is>
       </c>
       <c r="AE43" s="8" t="n"/>
@@ -5699,10 +5841,14 @@
       <c r="AT43" s="8" t="n"/>
       <c r="AU43" s="8" t="n"/>
       <c r="AV43" s="8" t="n"/>
-      <c r="AW43" s="8" t="n"/>
+      <c r="AW43" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX43" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Aluminium — category 'Other' not in current EPD database; carbon not estimated</t>
+          <t>[EXCLUDED] material: Aluminium hanging floor door stopper — category 'Other' not in current EPD database; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -5714,14 +5860,14 @@
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>34i</t>
+          <t>34 i</t>
         </is>
       </c>
       <c r="C44" s="8" t="n"/>
       <c r="D44" s="8" t="n"/>
       <c r="E44" s="8" t="inlineStr">
         <is>
-          <t>Providing and fixing steel glazed doors, windows and ventilators of standard rolled steel sections, joints mitred and welded with 15x3 mm lugs, 10 cm long, with steel lugs, embedded in cement concrete blocks 15x10x10 cm of 1:3:6 (1 cement : 3 coarse sand : 6 graded stone aggregate 20 mm nominal size) or with wooden plugs and screws or rawl plugs and screws or with fixing clips or with bolts and nuts as required, including providing and fixing of (Pin Head) 3mm thick glass panes with glazing clips and special metal sash putty of approved make complete including applying a priming coat of approved steel primer; excluding the cost of metal beading and other fitting except necessary hinges or pivots as required. i) Windows - side hung</t>
+          <t>Providing and fixing steel glazed doors, windows and ventilators of standard rolled steel sections, joints mitred and welded with 15x3 mm lugs, 10 cm long, with steel lugs, embedded in cement concrete blocks 15x10x10 cm of 1:3:6 (1 cement : 3 coarse sand : 6 graded stone aggregate 20 mm nominal size) or with wooden plugs and screws or rawl plugs and screws or with fixing clips or with bolts and nuts as required, including providing and fixing of (Pin Head) 3mm thick glass panes with glazing clips and special metal sash putty of approved make complete including applying a priming coat of approved steel primer; excluding the cost of metal beading and other fitting except necessary hinges or pivots as required. Windows - side hung</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
@@ -5736,12 +5882,12 @@
       </c>
       <c r="H44" s="8" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>Steel glazed windows</t>
         </is>
       </c>
       <c r="I44" s="8" t="inlineStr">
         <is>
-          <t>Steel, Glass, Cement, Coarse sand, Stone aggregate</t>
+          <t>Steel sections, Glass, Cement concrete, Putty, Steel primer</t>
         </is>
       </c>
       <c r="J44" s="8" t="inlineStr">
@@ -5810,7 +5956,7 @@
       <c r="AC44" s="8" t="n"/>
       <c r="AD44" s="8" t="inlineStr">
         <is>
-          <t>Steel &gt; Steel &gt; 1:3:6</t>
+          <t>Steel &gt; Steel glazed windows &gt; 1:3:6</t>
         </is>
       </c>
       <c r="AE44" s="8" t="n"/>
@@ -5833,10 +5979,14 @@
       <c r="AT44" s="8" t="n"/>
       <c r="AU44" s="8" t="n"/>
       <c r="AV44" s="8" t="n"/>
-      <c r="AW44" s="8" t="n"/>
+      <c r="AW44" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX44" s="8" t="inlineStr">
         <is>
-          <t>[OK] material: Steel — mass 266.12 kg [area × thickness (derived)] × 1.55 kgCO2e/kg = 412.48 kgCO2e — ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
+          <t>[OK] material: Steel glazed windows — mass 266.12 kg [area × thickness (derived)] × 1.55 kgCO2e/kg = 412.48 kgCO2e — ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
         </is>
       </c>
     </row>
@@ -5848,14 +5998,14 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>34ii</t>
+          <t>34 ii</t>
         </is>
       </c>
       <c r="C45" s="8" t="n"/>
       <c r="D45" s="8" t="n"/>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>Providing and fixing steel glazed doors, windows and ventilators of standard rolled steel sections, joints mitred and welded with 15x3 mm lugs, 10 cm long, with steel lugs, embedded in cement concrete blocks 15x10x10 cm of 1:3:6 (1 cement : 3 coarse sand : 6 graded stone aggregate 20 mm nominal size) or with wooden plugs and screws or rawl plugs and screws or with fixing clips or with bolts and nuts as required, including providing and fixing of (Pin Head) 3mm thick glass panes with glazing clips and special metal sash putty of approved make complete including applying a priming coat of approved steel primer; excluding the cost of metal beading and other fitting except necessary hinges or pivots as required. ii) Ventilators - centre hung</t>
+          <t>Providing and fixing steel glazed doors, windows and ventilators of standard rolled steel sections, joints mitred and welded with 15x3 mm lugs, 10 cm long, with steel lugs, embedded in cement concrete blocks 15x10x10 cm of 1:3:6 (1 cement : 3 coarse sand : 6 graded stone aggregate 20 mm nominal size) or with wooden plugs and screws or rawl plugs and screws or with fixing clips or with bolts and nuts as required, including providing and fixing of (Pin Head) 3mm thick glass panes with glazing clips and special metal sash putty of approved make complete including applying a priming coat of approved steel primer; excluding the cost of metal beading and other fitting except necessary hinges or pivots as required. Ventilators - centre hung</t>
         </is>
       </c>
       <c r="F45" s="8" t="inlineStr">
@@ -5870,12 +6020,12 @@
       </c>
       <c r="H45" s="8" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>Steel glazed ventilators</t>
         </is>
       </c>
       <c r="I45" s="8" t="inlineStr">
         <is>
-          <t>Steel, Glass, Cement, Coarse sand, Stone aggregate</t>
+          <t>Steel sections, Glass, Cement concrete, Putty, Steel primer</t>
         </is>
       </c>
       <c r="J45" s="8" t="inlineStr">
@@ -5944,7 +6094,7 @@
       <c r="AC45" s="8" t="n"/>
       <c r="AD45" s="8" t="inlineStr">
         <is>
-          <t>Steel &gt; Steel &gt; 1:3:6</t>
+          <t>Steel &gt; Steel glazed ventilators &gt; 1:3:6</t>
         </is>
       </c>
       <c r="AE45" s="8" t="n"/>
@@ -5967,10 +6117,14 @@
       <c r="AT45" s="8" t="n"/>
       <c r="AU45" s="8" t="n"/>
       <c r="AV45" s="8" t="n"/>
-      <c r="AW45" s="8" t="n"/>
+      <c r="AW45" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX45" s="8" t="inlineStr">
         <is>
-          <t>[OK] material: Steel — mass 23.55 kg [area × thickness (derived)] × 1.55 kgCO2e/kg = 36.5 kgCO2e — ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
+          <t>[OK] material: Steel glazed ventilators — mass 23.55 kg [area × thickness (derived)] × 1.55 kgCO2e/kg = 36.5 kgCO2e — ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
         </is>
       </c>
     </row>
@@ -6004,12 +6158,12 @@
       </c>
       <c r="H46" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>Mild steel casement window fasteners</t>
         </is>
       </c>
       <c r="I46" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>Oxidised mild steel, Machine screws</t>
         </is>
       </c>
       <c r="J46" s="8" t="inlineStr">
@@ -6062,7 +6216,7 @@
       <c r="AC46" s="8" t="n"/>
       <c r="AD46" s="8" t="inlineStr">
         <is>
-          <t>Steel &gt; Mild steel</t>
+          <t>Steel &gt; Mild steel casement window fasteners</t>
         </is>
       </c>
       <c r="AE46" s="8" t="n"/>
@@ -6083,10 +6237,14 @@
       <c r="AT46" s="8" t="n"/>
       <c r="AU46" s="8" t="n"/>
       <c r="AV46" s="8" t="n"/>
-      <c r="AW46" s="8" t="n"/>
+      <c r="AW46" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX46" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Mild steel — category 'Steel' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: Mild steel casement window fasteners — category 'Steel' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -6105,7 +6263,7 @@
       <c r="D47" s="8" t="n"/>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>Providing and fixing aluminium casement stays anodised transparent or dyed to requird colour and shade with with necessary welding and machine screws etc. complete.</t>
+          <t>Providing and fixing aluminium casement stays anodised transparent or dyed to required colour and shade with with necessary welding and machine screws etc. complete.</t>
         </is>
       </c>
       <c r="F47" s="8" t="inlineStr">
@@ -6120,12 +6278,12 @@
       </c>
       <c r="H47" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium casement stays</t>
         </is>
       </c>
       <c r="I47" s="8" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Aluminium, Screws</t>
         </is>
       </c>
       <c r="J47" s="8" t="inlineStr">
@@ -6174,7 +6332,7 @@
       <c r="AC47" s="8" t="n"/>
       <c r="AD47" s="8" t="inlineStr">
         <is>
-          <t>Other &gt; Aluminium</t>
+          <t>Other &gt; Aluminium casement stays</t>
         </is>
       </c>
       <c r="AE47" s="8" t="n"/>
@@ -6195,10 +6353,14 @@
       <c r="AT47" s="8" t="n"/>
       <c r="AU47" s="8" t="n"/>
       <c r="AV47" s="8" t="n"/>
-      <c r="AW47" s="8" t="n"/>
+      <c r="AW47" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX47" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Aluminium — category 'Other' not in current EPD database; carbon not estimated</t>
+          <t>[EXCLUDED] material: Aluminium casement stays — category 'Other' not in current EPD database; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -6232,12 +6394,12 @@
       </c>
       <c r="H48" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>MS Guard Flats</t>
         </is>
       </c>
       <c r="I48" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>Mild steel, Steel primer</t>
         </is>
       </c>
       <c r="J48" s="8" t="inlineStr">
@@ -6292,7 +6454,7 @@
       <c r="AC48" s="8" t="n"/>
       <c r="AD48" s="8" t="inlineStr">
         <is>
-          <t>Steel &gt; Mild steel</t>
+          <t>Steel &gt; MS Guard Flats</t>
         </is>
       </c>
       <c r="AE48" s="8" t="n"/>
@@ -6317,10 +6479,14 @@
       <c r="AT48" s="8" t="n"/>
       <c r="AU48" s="8" t="n"/>
       <c r="AV48" s="8" t="n"/>
-      <c r="AW48" s="8" t="n"/>
+      <c r="AW48" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX48" s="8" t="inlineStr">
         <is>
-          <t>[OK] material: Mild steel — mass 66.0 kg [direct weight] × 1.55 kgCO2e/kg = 102.3 kgCO2e — ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
+          <t>[OK] material: MS Guard Flats — mass 66.0 kg [direct weight] × 1.55 kgCO2e/kg = 102.3 kgCO2e — ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
         </is>
       </c>
     </row>
@@ -6354,12 +6520,12 @@
       </c>
       <c r="H49" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>T-Iron frames</t>
         </is>
       </c>
       <c r="I49" s="8" t="inlineStr">
         <is>
-          <t>Mild steel, Cement, Coarse sand, Stone aggregate</t>
+          <t>Mild steel Tee sections, Cement concrete, Steel primer</t>
         </is>
       </c>
       <c r="J49" s="8" t="inlineStr">
@@ -6418,7 +6584,7 @@
       <c r="AC49" s="8" t="n"/>
       <c r="AD49" s="8" t="inlineStr">
         <is>
-          <t>Steel &gt; Mild steel &gt; 1:3:6</t>
+          <t>Steel &gt; T-Iron frames &gt; 1:3:6</t>
         </is>
       </c>
       <c r="AE49" s="8" t="n"/>
@@ -6439,10 +6605,14 @@
       <c r="AT49" s="8" t="n"/>
       <c r="AU49" s="8" t="n"/>
       <c r="AV49" s="8" t="n"/>
-      <c r="AW49" s="8" t="n"/>
+      <c r="AW49" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX49" s="8" t="inlineStr">
         <is>
-          <t>[OK] material: Mild steel — mass 187.0 kg [direct weight] × 1.55 kgCO2e/kg = 289.85 kgCO2e — ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
+          <t>[OK] material: T-Iron frames — mass 187.0 kg [direct weight] × 1.55 kgCO2e/kg = 289.85 kgCO2e — ICE Database V4.0 (Steel Open Sections) via NZBG Guide V1.0</t>
         </is>
       </c>
     </row>
@@ -6471,17 +6641,17 @@
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Structural</t>
         </is>
       </c>
       <c r="H50" s="8" t="inlineStr">
         <is>
-          <t>Mild steel bar</t>
+          <t>MS fan clamp</t>
         </is>
       </c>
       <c r="I50" s="8" t="inlineStr">
         <is>
-          <t>Mild steel</t>
+          <t>Mild steel bar, Paint</t>
         </is>
       </c>
       <c r="J50" s="8" t="inlineStr">
@@ -6534,7 +6704,7 @@
       <c r="AC50" s="8" t="n"/>
       <c r="AD50" s="8" t="inlineStr">
         <is>
-          <t>Steel &gt; Mild steel bar</t>
+          <t>Steel &gt; MS fan clamp</t>
         </is>
       </c>
       <c r="AE50" s="8" t="n"/>
@@ -6557,10 +6727,14 @@
       </c>
       <c r="AU50" s="8" t="n"/>
       <c r="AV50" s="8" t="n"/>
-      <c r="AW50" s="8" t="n"/>
+      <c r="AW50" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX50" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Mild steel bar — category 'Steel' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: MS fan clamp — category 'Steel' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -6594,7 +6768,7 @@
       </c>
       <c r="H51" s="8" t="inlineStr">
         <is>
-          <t>Cement concrete</t>
+          <t>Cement concrete flooring</t>
         </is>
       </c>
       <c r="I51" s="8" t="inlineStr">
@@ -6672,7 +6846,7 @@
       <c r="AC51" s="8" t="n"/>
       <c r="AD51" s="8" t="inlineStr">
         <is>
-          <t>Concrete &gt; Cement concrete &gt; M15</t>
+          <t>Concrete &gt; Cement concrete flooring &gt; M15</t>
         </is>
       </c>
       <c r="AE51" s="8" t="n"/>
@@ -6695,10 +6869,14 @@
       <c r="AT51" s="8" t="n"/>
       <c r="AU51" s="8" t="n"/>
       <c r="AV51" s="8" t="n"/>
-      <c r="AW51" s="8" t="n"/>
+      <c r="AW51" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX51" s="8" t="inlineStr">
         <is>
-          <t>[OK] material: Cement concrete — mass 6528.0 kg [area × thickness (derived)] × 0.149 kgCO2e/kg = 972.67 kgCO2e — ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
+          <t>[OK] material: Cement concrete flooring — mass 6528.0 kg [area × thickness (derived)] × 0.149 kgCO2e/kg = 972.67 kgCO2e — ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
         </is>
       </c>
     </row>
@@ -6717,7 +6895,7 @@
       <c r="D52" s="8" t="n"/>
       <c r="E52" s="8" t="inlineStr">
         <is>
-          <t>18 mm thick cement plastesr skirting (upto 30 cm height) with cement mortar 1:3 (1 cement : 3 coarse sand) finished with a floating coat of neat cement including rounding of junctions with floors.</t>
+          <t>18 mm thick cement plaster skirting (upto 30 cm height) with cement mortar 1:3 (1 cement : 3 coarse sand) finished with a floating coat of neat cement including rounding of junctions with floors.</t>
         </is>
       </c>
       <c r="F52" s="8" t="inlineStr">
@@ -6732,7 +6910,7 @@
       </c>
       <c r="H52" s="8" t="inlineStr">
         <is>
-          <t>Cement plaster</t>
+          <t>Cement plaster skirting</t>
         </is>
       </c>
       <c r="I52" s="8" t="inlineStr">
@@ -6806,7 +6984,7 @@
       <c r="AC52" s="8" t="n"/>
       <c r="AD52" s="8" t="inlineStr">
         <is>
-          <t>Plaster &gt; Cement plaster &gt; 1:3</t>
+          <t>Plaster &gt; Cement plaster skirting &gt; 1:3</t>
         </is>
       </c>
       <c r="AE52" s="8" t="n"/>
@@ -6831,10 +7009,14 @@
       <c r="AT52" s="8" t="n"/>
       <c r="AU52" s="8" t="n"/>
       <c r="AV52" s="8" t="n"/>
-      <c r="AW52" s="8" t="n"/>
+      <c r="AW52" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX52" s="8" t="inlineStr">
         <is>
-          <t>[OK] material: Cement plaster — mass 376.2 kg [area × thickness (derived)] × 0.163 kgCO2e/kg = 61.32 kgCO2e — ICE Database V4.0 (Cement Mortar 1:3, general) via NZBG Guide V1.0</t>
+          <t>[OK] material: Cement plaster skirting — mass 376.2 kg [area × thickness (derived)] × 0.163 kgCO2e/kg = 61.32 kgCO2e — ICE Database V4.0 (Cement Mortar 1:3, general) via NZBG Guide V1.0</t>
         </is>
       </c>
     </row>
@@ -6873,7 +7055,7 @@
       </c>
       <c r="I53" s="8" t="inlineStr">
         <is>
-          <t>Cement, Coarse sand, Stone aggregate, Marble chips, Marble powder</t>
+          <t>Marble chips, Cement, Coarse sand, Stone aggregate, Marble powder, Pigment</t>
         </is>
       </c>
       <c r="J53" s="8" t="inlineStr">
@@ -6969,7 +7151,11 @@
       <c r="AT53" s="8" t="n"/>
       <c r="AU53" s="8" t="n"/>
       <c r="AV53" s="8" t="n"/>
-      <c r="AW53" s="8" t="n"/>
+      <c r="AW53" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX53" s="8" t="inlineStr">
         <is>
           <t>[OK] material: Marble chips flooring — mass 864.0 kg [area × thickness (derived)] × 0.149 kgCO2e/kg = 128.74 kgCO2e — ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M15 inferred from nominal mix 1:2:4 (IS 456)</t>
@@ -7085,7 +7271,11 @@
       <c r="AT54" s="8" t="n"/>
       <c r="AU54" s="8" t="n"/>
       <c r="AV54" s="8" t="n"/>
-      <c r="AW54" s="8" t="n"/>
+      <c r="AW54" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX54" s="8" t="inlineStr">
         <is>
           <t>[EXCLUDED] material: Glass strips — category 'Other' not in current EPD database; carbon not estimated</t>
@@ -7107,7 +7297,7 @@
       <c r="D55" s="8" t="n"/>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t>Painting top of roofs with bitumen of approved quality at 17 Kg. per 10 square metre impregnated with a coat of coarse sand at 3/2 60 dm per 10 m including cleaning the slab surface with brushes and finally with a piece of cloth lightly soaked in kerosene oil complete with residual type petroleum bitumen of penetration 80/100.</t>
+          <t>Painting top of roofs with bitumen of approved quality at 17 Kg. per 10 square metre impregnated with a coat of coarse sand at 3/60 dm^2 per 10 m^2 including cleaning the slab surface with brushes and finally with a piece of cloth lightly soaked in kerosene oil complete with residual type petroleum bitumen of penetration 80/100.</t>
         </is>
       </c>
       <c r="F55" s="8" t="inlineStr">
@@ -7122,7 +7312,7 @@
       </c>
       <c r="H55" s="8" t="inlineStr">
         <is>
-          <t>Bitumen</t>
+          <t>Bitumen painting</t>
         </is>
       </c>
       <c r="I55" s="8" t="inlineStr">
@@ -7180,7 +7370,7 @@
       <c r="AC55" s="8" t="n"/>
       <c r="AD55" s="8" t="inlineStr">
         <is>
-          <t>Paint/Finish &gt; Bitumen</t>
+          <t>Paint/Finish &gt; Bitumen painting</t>
         </is>
       </c>
       <c r="AE55" s="8" t="n"/>
@@ -7201,10 +7391,14 @@
       <c r="AT55" s="8" t="n"/>
       <c r="AU55" s="8" t="n"/>
       <c r="AV55" s="8" t="n"/>
-      <c r="AW55" s="8" t="n"/>
+      <c r="AW55" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX55" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Bitumen — category 'Paint/Finish' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: Bitumen painting — category 'Paint/Finish' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -7238,12 +7432,12 @@
       </c>
       <c r="H56" s="8" t="inlineStr">
         <is>
-          <t>Lime concrete</t>
+          <t>Lime concrete terracing</t>
         </is>
       </c>
       <c r="I56" s="8" t="inlineStr">
         <is>
-          <t>Lime putty, Surkhi, Brick aggregate, Brick tiles, Cement, Fine sand</t>
+          <t>Brick aggregate, Lime putty, Surkhi, Gur, Belgiri, Brick tiles, Cement, Fine sand, Crude oil</t>
         </is>
       </c>
       <c r="J56" s="8" t="inlineStr">
@@ -7312,7 +7506,7 @@
       <c r="AC56" s="8" t="n"/>
       <c r="AD56" s="8" t="inlineStr">
         <is>
-          <t>Concrete &gt; Lime concrete &gt; 1:2</t>
+          <t>Concrete &gt; Lime concrete terracing &gt; 1:2</t>
         </is>
       </c>
       <c r="AE56" s="8" t="n"/>
@@ -7335,10 +7529,14 @@
       <c r="AT56" s="8" t="n"/>
       <c r="AU56" s="8" t="n"/>
       <c r="AV56" s="8" t="n"/>
-      <c r="AW56" s="8" t="n"/>
+      <c r="AW56" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX56" s="8" t="inlineStr">
         <is>
-          <t>[OK] material: Lime concrete — mass 15600.0 kg [area × thickness (derived)] × 0.149 kgCO2e/kg = 2324.4 kgCO2e — ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0</t>
+          <t>[OK] material: Lime concrete terracing — mass 15600.0 kg [area × thickness (derived)] × 0.149 kgCO2e/kg = 2324.4 kgCO2e — ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0</t>
         </is>
       </c>
     </row>
@@ -7367,7 +7565,7 @@
       </c>
       <c r="G57" s="8" t="inlineStr">
         <is>
-          <t>Finishes</t>
+          <t>Civil &amp; Sitework</t>
         </is>
       </c>
       <c r="H57" s="8" t="inlineStr">
@@ -7473,7 +7671,11 @@
       <c r="AT57" s="8" t="n"/>
       <c r="AU57" s="8" t="n"/>
       <c r="AV57" s="8" t="n"/>
-      <c r="AW57" s="8" t="n"/>
+      <c r="AW57" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX57" s="8" t="inlineStr">
         <is>
           <t>[OK] material: Burnt clay tiles — mass 1440.0 kg [area × thickness (derived)] × 0.213 kgCO2e/kg = 306.72 kgCO2e — ICE Database V4.0 (Brick Clay) via NZBG Guide V1.0</t>
@@ -7510,7 +7712,7 @@
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>Cement concrete</t>
+          <t>Cement concrete gola</t>
         </is>
       </c>
       <c r="I58" s="8" t="inlineStr">
@@ -7576,7 +7778,7 @@
       <c r="AC58" s="8" t="n"/>
       <c r="AD58" s="8" t="inlineStr">
         <is>
-          <t>Concrete &gt; Cement concrete &gt; M10</t>
+          <t>Concrete &gt; Cement concrete gola &gt; M10</t>
         </is>
       </c>
       <c r="AE58" s="8" t="n"/>
@@ -7601,10 +7803,14 @@
       <c r="AT58" s="8" t="n"/>
       <c r="AU58" s="8" t="n"/>
       <c r="AV58" s="8" t="n"/>
-      <c r="AW58" s="8" t="n"/>
+      <c r="AW58" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX58" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Cement concrete — category 'Concrete' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: Cement concrete gola — category 'Concrete' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -7638,7 +7844,7 @@
       </c>
       <c r="H59" s="8" t="inlineStr">
         <is>
-          <t>Cement concrete</t>
+          <t>Cement concrete khurras</t>
         </is>
       </c>
       <c r="I59" s="8" t="inlineStr">
@@ -7704,7 +7910,7 @@
       <c r="AC59" s="8" t="n"/>
       <c r="AD59" s="8" t="inlineStr">
         <is>
-          <t>Concrete &gt; Cement concrete &gt; M15</t>
+          <t>Concrete &gt; Cement concrete khurras &gt; M15</t>
         </is>
       </c>
       <c r="AE59" s="8" t="n"/>
@@ -7731,10 +7937,14 @@
       <c r="AT59" s="8" t="n"/>
       <c r="AU59" s="8" t="n"/>
       <c r="AV59" s="8" t="n"/>
-      <c r="AW59" s="8" t="n"/>
+      <c r="AW59" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX59" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Cement concrete — category 'Concrete' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: Cement concrete khurras — category 'Concrete' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -7768,12 +7978,12 @@
       </c>
       <c r="H60" s="8" t="inlineStr">
         <is>
-          <t>Cast iron pipe</t>
+          <t>CI rain water pipe</t>
         </is>
       </c>
       <c r="I60" s="8" t="inlineStr">
         <is>
-          <t>Cast iron, Cement, Fine sand, Spun yarn</t>
+          <t>Cast Iron, Spun yarn, Cement, Fine sand</t>
         </is>
       </c>
       <c r="J60" s="8" t="inlineStr">
@@ -7826,7 +8036,7 @@
       <c r="AC60" s="8" t="n"/>
       <c r="AD60" s="8" t="inlineStr">
         <is>
-          <t>Other &gt; Cast iron pipe &gt; 1:2</t>
+          <t>Other &gt; CI rain water pipe &gt; 1:2</t>
         </is>
       </c>
       <c r="AE60" s="8" t="n"/>
@@ -7849,10 +8059,14 @@
       </c>
       <c r="AU60" s="8" t="n"/>
       <c r="AV60" s="8" t="n"/>
-      <c r="AW60" s="8" t="n"/>
+      <c r="AW60" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX60" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Cast iron pipe — category 'Other' not in current EPD database; carbon not estimated</t>
+          <t>[EXCLUDED] material: CI rain water pipe — category 'Other' not in current EPD database; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -7886,7 +8100,7 @@
       </c>
       <c r="H61" s="8" t="inlineStr">
         <is>
-          <t>Mild steel holderbat clamp</t>
+          <t>MS holderbat clamps</t>
         </is>
       </c>
       <c r="I61" s="8" t="inlineStr">
@@ -7948,7 +8162,7 @@
       <c r="AC61" s="8" t="n"/>
       <c r="AD61" s="8" t="inlineStr">
         <is>
-          <t>Steel &gt; Mild steel holderbat clamp &gt; 1:2:4</t>
+          <t>Steel &gt; MS holderbat clamps &gt; 1:2:4</t>
         </is>
       </c>
       <c r="AE61" s="8" t="n"/>
@@ -7961,9 +8175,15 @@
       <c r="AL61" s="8" t="n"/>
       <c r="AM61" s="8" t="n"/>
       <c r="AN61" s="8" t="n"/>
-      <c r="AO61" s="8" t="n"/>
-      <c r="AP61" s="8" t="n"/>
-      <c r="AQ61" s="8" t="n"/>
+      <c r="AO61" s="17" t="n">
+        <v>100</v>
+      </c>
+      <c r="AP61" s="17" t="n">
+        <v>100</v>
+      </c>
+      <c r="AQ61" s="17" t="n">
+        <v>100</v>
+      </c>
       <c r="AR61" s="8" t="n"/>
       <c r="AS61" s="8" t="n"/>
       <c r="AT61" s="17" t="n">
@@ -7971,10 +8191,14 @@
       </c>
       <c r="AU61" s="8" t="n"/>
       <c r="AV61" s="8" t="n"/>
-      <c r="AW61" s="8" t="n"/>
+      <c r="AW61" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX61" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Mild steel holderbat clamp — category 'Steel' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: MS holderbat clamps — category 'Steel' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -7986,14 +8210,14 @@
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>51i</t>
+          <t>51 i</t>
         </is>
       </c>
       <c r="C62" s="8" t="n"/>
       <c r="D62" s="8" t="n"/>
       <c r="E62" s="8" t="inlineStr">
         <is>
-          <t>Providing and fixing on wall face CI accessories for rain water pipes including filling the joints with spun yarn soaked in neat cement slurry and cement mortar 1:2 (1 cement : 2 fine sand) i) CI plain head 100 mm dia</t>
+          <t>Providing and fixing on wall face CI accessories for rain water pipes including filling the joints with spun yarn soaked in neat cement slurry and cement mortar 1:2 (1 cement : 2 fine sand) CI plain head 100 mm dia</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
@@ -8008,12 +8232,12 @@
       </c>
       <c r="H62" s="8" t="inlineStr">
         <is>
-          <t>Cast iron</t>
+          <t>CI plain head</t>
         </is>
       </c>
       <c r="I62" s="8" t="inlineStr">
         <is>
-          <t>Cast iron, Cement, Fine sand</t>
+          <t>Cast iron, Spun yarn, Cement, Fine sand</t>
         </is>
       </c>
       <c r="J62" s="8" t="inlineStr">
@@ -8066,7 +8290,7 @@
       <c r="AC62" s="8" t="n"/>
       <c r="AD62" s="8" t="inlineStr">
         <is>
-          <t>Other &gt; Cast iron &gt; 1:2</t>
+          <t>Other &gt; CI plain head &gt; 1:2</t>
         </is>
       </c>
       <c r="AE62" s="8" t="n"/>
@@ -8089,10 +8313,14 @@
       </c>
       <c r="AU62" s="8" t="n"/>
       <c r="AV62" s="8" t="n"/>
-      <c r="AW62" s="8" t="n"/>
+      <c r="AW62" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX62" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Cast iron — category 'Other' not in current EPD database; carbon not estimated</t>
+          <t>[EXCLUDED] material: CI plain head — category 'Other' not in current EPD database; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -8104,14 +8332,14 @@
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>51ii</t>
+          <t>51 ii</t>
         </is>
       </c>
       <c r="C63" s="8" t="n"/>
       <c r="D63" s="8" t="n"/>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t>Providing and fixing on wall face CI accessories for rain water pipes including filling the joints with spun yarn soaked in neat cement slurry and cement mortar 1:2 (1 cement : 2 fine sand) ii) CI plain shoe - 100 mm dia</t>
+          <t>Providing and fixing on wall face CI accessories for rain water pipes including filling the joints with spun yarn soaked in neat cement slurry and cement mortar 1:2 (1 cement : 2 fine sand) CI plain shoe - 100 mm dia</t>
         </is>
       </c>
       <c r="F63" s="8" t="inlineStr">
@@ -8126,12 +8354,12 @@
       </c>
       <c r="H63" s="8" t="inlineStr">
         <is>
-          <t>Cast iron</t>
+          <t>CI plain shoe</t>
         </is>
       </c>
       <c r="I63" s="8" t="inlineStr">
         <is>
-          <t>Cast iron, Cement, Fine sand</t>
+          <t>Cast iron, Spun yarn, Cement, Fine sand</t>
         </is>
       </c>
       <c r="J63" s="8" t="inlineStr">
@@ -8184,7 +8412,7 @@
       <c r="AC63" s="8" t="n"/>
       <c r="AD63" s="8" t="inlineStr">
         <is>
-          <t>Other &gt; Cast iron &gt; 1:2</t>
+          <t>Other &gt; CI plain shoe &gt; 1:2</t>
         </is>
       </c>
       <c r="AE63" s="8" t="n"/>
@@ -8207,10 +8435,14 @@
       </c>
       <c r="AU63" s="8" t="n"/>
       <c r="AV63" s="8" t="n"/>
-      <c r="AW63" s="8" t="n"/>
+      <c r="AW63" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX63" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Cast iron — category 'Other' not in current EPD database; carbon not estimated</t>
+          <t>[EXCLUDED] material: CI plain shoe — category 'Other' not in current EPD database; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -8222,14 +8454,14 @@
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>51iii</t>
+          <t>51 iii</t>
         </is>
       </c>
       <c r="C64" s="8" t="n"/>
       <c r="D64" s="8" t="n"/>
       <c r="E64" s="8" t="inlineStr">
         <is>
-          <t>Providing and fixing on wall face CI accessories for rain water pipes including filling the joints with spun yarn soaked in neat cement slurry and cement mortar 1:2 (1 cement : 2 fine sand) iii) CI plain bend - 100 mm dia</t>
+          <t>Providing and fixing on wall face CI accessories for rain water pipes including filling the joints with spun yarn soaked in neat cement slurry and cement mortar 1:2 (1 cement : 2 fine sand) CI plain bend - 100 mm dia</t>
         </is>
       </c>
       <c r="F64" s="8" t="inlineStr">
@@ -8244,12 +8476,12 @@
       </c>
       <c r="H64" s="8" t="inlineStr">
         <is>
-          <t>Cast iron</t>
+          <t>CI plain bend</t>
         </is>
       </c>
       <c r="I64" s="8" t="inlineStr">
         <is>
-          <t>Cast iron, Cement, Fine sand</t>
+          <t>Cast iron, Spun yarn, Cement, Fine sand</t>
         </is>
       </c>
       <c r="J64" s="8" t="inlineStr">
@@ -8302,7 +8534,7 @@
       <c r="AC64" s="8" t="n"/>
       <c r="AD64" s="8" t="inlineStr">
         <is>
-          <t>Other &gt; Cast iron &gt; 1:2</t>
+          <t>Other &gt; CI plain bend &gt; 1:2</t>
         </is>
       </c>
       <c r="AE64" s="8" t="n"/>
@@ -8325,10 +8557,14 @@
       </c>
       <c r="AU64" s="8" t="n"/>
       <c r="AV64" s="8" t="n"/>
-      <c r="AW64" s="8" t="n"/>
+      <c r="AW64" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX64" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Cast iron — category 'Other' not in current EPD database; carbon not estimated</t>
+          <t>[EXCLUDED] material: CI plain bend — category 'Other' not in current EPD database; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -8459,7 +8695,11 @@
       <c r="AT65" s="8" t="n"/>
       <c r="AU65" s="8" t="n"/>
       <c r="AV65" s="8" t="n"/>
-      <c r="AW65" s="8" t="n"/>
+      <c r="AW65" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX65" s="8" t="inlineStr">
         <is>
           <t>[OK] material: Cement plaster — mass 5016.0 kg [area × thickness (derived)] × 0.163 kgCO2e/kg = 817.61 kgCO2e — ICE Database V4.0 (Cement Mortar 1:3, general) via NZBG Guide V1.0</t>
@@ -8593,7 +8833,11 @@
       <c r="AT66" s="8" t="n"/>
       <c r="AU66" s="8" t="n"/>
       <c r="AV66" s="8" t="n"/>
-      <c r="AW66" s="8" t="n"/>
+      <c r="AW66" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX66" s="8" t="inlineStr">
         <is>
           <t>[OK] material: Cement plaster — mass 6270.0 kg [area × thickness (derived)] × 0.163 kgCO2e/kg = 1022.01 kgCO2e — ICE Database V4.0 (Cement Mortar 1:3, general) via NZBG Guide V1.0</t>
@@ -8635,7 +8879,7 @@
       </c>
       <c r="I67" s="8" t="inlineStr">
         <is>
-          <t>Cement, Fine sand, Lime</t>
+          <t>Cement, Fine sand, Lime wash</t>
         </is>
       </c>
       <c r="J67" s="8" t="inlineStr">
@@ -8727,7 +8971,11 @@
       <c r="AT67" s="8" t="n"/>
       <c r="AU67" s="8" t="n"/>
       <c r="AV67" s="8" t="n"/>
-      <c r="AW67" s="8" t="n"/>
+      <c r="AW67" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX67" s="8" t="inlineStr">
         <is>
           <t>[OK] material: Cement plaster — mass 216.6 kg [area × thickness (derived)] × 0.163 kgCO2e/kg = 35.31 kgCO2e — ICE Database V4.0 (Cement Mortar 1:3, general) via NZBG Guide V1.0</t>
@@ -8764,7 +9012,7 @@
       </c>
       <c r="H68" s="8" t="inlineStr">
         <is>
-          <t>Terrazzo plaster</t>
+          <t>Terrazzo plaster dado</t>
         </is>
       </c>
       <c r="I68" s="8" t="inlineStr">
@@ -8838,7 +9086,7 @@
       <c r="AC68" s="8" t="n"/>
       <c r="AD68" s="8" t="inlineStr">
         <is>
-          <t>Plaster &gt; Terrazzo plaster &gt; 1:3</t>
+          <t>Plaster &gt; Terrazzo plaster dado &gt; 1:3</t>
         </is>
       </c>
       <c r="AE68" s="8" t="n"/>
@@ -8861,10 +9109,14 @@
       <c r="AT68" s="8" t="n"/>
       <c r="AU68" s="8" t="n"/>
       <c r="AV68" s="8" t="n"/>
-      <c r="AW68" s="8" t="n"/>
+      <c r="AW68" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX68" s="8" t="inlineStr">
         <is>
-          <t>[OK] material: Terrazzo plaster — mass 684.0 kg [area × thickness (derived)] × 0.163 kgCO2e/kg = 111.49 kgCO2e — ICE Database V4.0 (Cement Mortar 1:3, general) via NZBG Guide V1.0</t>
+          <t>[OK] material: Terrazzo plaster dado — mass 684.0 kg [area × thickness (derived)] × 0.163 kgCO2e/kg = 111.49 kgCO2e — ICE Database V4.0 (Cement Mortar 1:3, general) via NZBG Guide V1.0</t>
         </is>
       </c>
     </row>
@@ -8898,7 +9150,7 @@
       </c>
       <c r="H69" s="8" t="inlineStr">
         <is>
-          <t>Cement mortar plaster</t>
+          <t>Cement plaster</t>
         </is>
       </c>
       <c r="I69" s="8" t="inlineStr">
@@ -8960,7 +9212,7 @@
       <c r="AC69" s="8" t="n"/>
       <c r="AD69" s="8" t="inlineStr">
         <is>
-          <t>Plaster &gt; Cement mortar plaster &gt; 1:3</t>
+          <t>Plaster &gt; Cement plaster &gt; 1:3</t>
         </is>
       </c>
       <c r="AE69" s="8" t="n"/>
@@ -8981,10 +9233,14 @@
       <c r="AT69" s="8" t="n"/>
       <c r="AU69" s="8" t="n"/>
       <c r="AV69" s="8" t="n"/>
-      <c r="AW69" s="8" t="n"/>
+      <c r="AW69" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX69" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Cement mortar plaster — category 'Plaster' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: Cement plaster — category 'Plaster' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -9018,7 +9274,7 @@
       </c>
       <c r="H70" s="8" t="inlineStr">
         <is>
-          <t>Lime wash</t>
+          <t>White wash</t>
         </is>
       </c>
       <c r="I70" s="8" t="inlineStr">
@@ -9076,7 +9332,7 @@
       <c r="AC70" s="8" t="n"/>
       <c r="AD70" s="8" t="inlineStr">
         <is>
-          <t>Paint/Finish &gt; Lime wash</t>
+          <t>Paint/Finish &gt; White wash</t>
         </is>
       </c>
       <c r="AE70" s="8" t="n"/>
@@ -9097,10 +9353,14 @@
       <c r="AT70" s="8" t="n"/>
       <c r="AU70" s="8" t="n"/>
       <c r="AV70" s="8" t="n"/>
-      <c r="AW70" s="8" t="n"/>
+      <c r="AW70" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX70" s="8" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Lime wash — category 'Paint/Finish' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: White wash — category 'Paint/Finish' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -9139,7 +9399,7 @@
       </c>
       <c r="I71" s="8" t="inlineStr">
         <is>
-          <t>Lime</t>
+          <t>Lime, Colour wash pigment</t>
         </is>
       </c>
       <c r="J71" s="8" t="inlineStr">
@@ -9213,7 +9473,11 @@
       <c r="AT71" s="8" t="n"/>
       <c r="AU71" s="8" t="n"/>
       <c r="AV71" s="8" t="n"/>
-      <c r="AW71" s="8" t="n"/>
+      <c r="AW71" s="8" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX71" s="8" t="inlineStr">
         <is>
           <t>[EXCLUDED] material: Colour wash — category 'Paint/Finish' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
@@ -9248,12 +9512,12 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Primer</t>
+          <t>Wood primer</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Primer</t>
+          <t>Pink/gray primer</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -9295,12 +9559,17 @@
       </c>
       <c r="AD72" t="inlineStr">
         <is>
-          <t>Paint/Finish &gt; Primer</t>
+          <t>Paint/Finish &gt; Wood primer</t>
+        </is>
+      </c>
+      <c r="AW72" t="inlineStr">
+        <is>
+          <t>INR</t>
         </is>
       </c>
       <c r="AX72" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Primer — category 'Paint/Finish' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: Wood primer — category 'Paint/Finish' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -9332,12 +9601,12 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Zinc chromate primer</t>
+          <t>Zinc chromate yellow primer</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Zinc chromate primer</t>
+          <t>Zinc chromate yellow primer</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -9379,12 +9648,17 @@
       </c>
       <c r="AD73" t="inlineStr">
         <is>
-          <t>Paint/Finish &gt; Zinc chromate primer</t>
+          <t>Paint/Finish &gt; Zinc chromate yellow primer</t>
+        </is>
+      </c>
+      <c r="AW73" t="inlineStr">
+        <is>
+          <t>INR</t>
         </is>
       </c>
       <c r="AX73" t="inlineStr">
         <is>
-          <t>[EXCLUDED] material: Zinc chromate primer — category 'Paint/Finish' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
+          <t>[EXCLUDED] material: Zinc chromate yellow primer — category 'Paint/Finish' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
         </is>
       </c>
     </row>
@@ -9421,7 +9695,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Bitumastic paint, Zinc chromate primer</t>
+          <t>Bitumastic paint, Zinc chromate yellow primer</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -9469,6 +9743,11 @@
       <c r="AT74" s="18" t="n">
         <v>100</v>
       </c>
+      <c r="AW74" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX74" t="inlineStr">
         <is>
           <t>[EXCLUDED] material: Bitumastic paint — category 'Paint/Finish' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
@@ -9553,6 +9832,11 @@
           <t>Paint/Finish &gt; Synthetic enamel paint</t>
         </is>
       </c>
+      <c r="AW75" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX75" t="inlineStr">
         <is>
           <t>[EXCLUDED] material: Synthetic enamel paint — category 'Paint/Finish' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
@@ -9592,7 +9876,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>French spirit polish, Wood filler</t>
+          <t>French spirit, Wood filler</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -9637,6 +9921,11 @@
           <t>Paint/Finish &gt; French spirit polish</t>
         </is>
       </c>
+      <c r="AW76" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX76" t="inlineStr">
         <is>
           <t>[EXCLUDED] material: French spirit polish — category 'Paint/Finish' has an EPD factor but no usable weight/volume figure was available to compute mass; carbon not estimated</t>
@@ -9671,7 +9960,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Cement concrete</t>
+          <t>Cement concrete plinth protection</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -9744,15 +10033,20 @@
       </c>
       <c r="AD77" t="inlineStr">
         <is>
-          <t>Concrete &gt; Cement concrete &gt; M10</t>
+          <t>Concrete &gt; Cement concrete plinth protection &gt; M10</t>
         </is>
       </c>
       <c r="AR77" s="18" t="n">
         <v>50</v>
       </c>
+      <c r="AW77" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="AX77" t="inlineStr">
         <is>
-          <t>[OK] material: Cement concrete — mass 4152.0 kg [area × thickness (derived)] × 0.149 kgCO2e/kg = 618.65 kgCO2e — ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M10 inferred from nominal mix 1:3:6 (IS 456)</t>
+          <t>[OK] material: Cement concrete plinth protection — mass 4152.0 kg [area × thickness (derived)] × 0.149 kgCO2e/kg = 618.65 kgCO2e — ICE Database V4.1 (Concrete C35/45) via NZBG Guide V1.0; Grade M10 inferred from nominal mix 1:3:6 (IS 456)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix build file error
</commit_message>
<xml_diff>
--- a/output/passport_filled.xlsx
+++ b/output/passport_filled.xlsx
@@ -1164,7 +1164,7 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - I, Earth Work</t>
+          <t>Sub-Head - VII, Flooring &amp; Roof Treatment</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - I, Earth Work</t>
+          <t>Sub-Head - VII, Flooring &amp; Roof Treatment</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - II, Cement Concrete Work</t>
+          <t>Sub-Head - VII, Flooring &amp; Roof Treatment</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - II, Cement Concrete Work</t>
+          <t>Sub-Head - VII, Flooring &amp; Roof Treatment</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - II, Cement Concrete Work</t>
+          <t>Sub-Head - VII, Flooring &amp; Roof Treatment</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - II, Cement Concrete Work</t>
+          <t>Sub-Head - VII, Flooring &amp; Roof Treatment</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
@@ -2816,7 +2816,7 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - III, R.C.C. Work</t>
+          <t>Sub-Head - VII, Flooring &amp; Roof Treatment</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - III, R.C.C. Work</t>
+          <t>Schedule 'A'</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
@@ -3048,7 +3048,7 @@
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - III, R.C.C. Work</t>
+          <t>Schedule 'A'</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - III, R.C.C. Work</t>
+          <t>Schedule 'A'</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
@@ -3280,7 +3280,7 @@
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - III, R.C.C. Work</t>
+          <t>Schedule 'A'</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
@@ -4526,7 +4526,7 @@
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - V, Wood Work</t>
+          <t>Sub-Head - VI, Steel &amp; Aluminium Fittings</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="F44" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - VI, Steel &amp; Aluminium Fittings</t>
+          <t>Sub-Head - V, Wood Work</t>
         </is>
       </c>
       <c r="G44" s="8" t="inlineStr">
@@ -6010,7 +6010,7 @@
       </c>
       <c r="F45" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - VI, Steel &amp; Aluminium Fittings</t>
+          <t>Sub-Head - V, Wood Work</t>
         </is>
       </c>
       <c r="G45" s="8" t="inlineStr">
@@ -6510,7 +6510,7 @@
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - VI, Steel &amp; Aluminium Fittings</t>
+          <t>Sub-Head - V, Wood Work</t>
         </is>
       </c>
       <c r="G49" s="8" t="inlineStr">
@@ -6636,7 +6636,7 @@
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - VI, Steel &amp; Aluminium Fittings</t>
+          <t>Sub-Head - III, R.C.C. Work</t>
         </is>
       </c>
       <c r="G50" s="8" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="F55" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - VII, Flooring &amp; Roof Treatment</t>
+          <t>Sub-Head - X, White/Colour Washing &amp; Painting</t>
         </is>
       </c>
       <c r="G55" s="8" t="inlineStr">
@@ -7560,7 +7560,7 @@
       </c>
       <c r="F57" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - VII, Flooring &amp; Roof Treatment</t>
+          <t>Sub-Head - IV, Brick Work</t>
         </is>
       </c>
       <c r="G57" s="8" t="inlineStr">
@@ -7702,7 +7702,7 @@
       </c>
       <c r="F58" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - VII, Flooring &amp; Roof Treatment</t>
+          <t>Sub-Head - II, Cement Concrete Work</t>
         </is>
       </c>
       <c r="G58" s="8" t="inlineStr">
@@ -7834,7 +7834,7 @@
       </c>
       <c r="F59" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - VII, Flooring &amp; Roof Treatment</t>
+          <t>Sub-Head - IX, Plastering</t>
         </is>
       </c>
       <c r="G59" s="8" t="inlineStr">
@@ -8090,7 +8090,7 @@
       </c>
       <c r="F61" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - VIII, Sanitary Installation (Rain Water Pipes)</t>
+          <t>Sub-Head - VI, Steel &amp; Aluminium Fittings</t>
         </is>
       </c>
       <c r="G61" s="8" t="inlineStr">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="F67" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - IX, Plastering</t>
+          <t>Sub-Head - III, R.C.C. Work</t>
         </is>
       </c>
       <c r="G67" s="8" t="inlineStr">
@@ -9002,7 +9002,7 @@
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - IX, Plastering</t>
+          <t>Sub-Head - VII, Flooring &amp; Roof Treatment</t>
         </is>
       </c>
       <c r="G68" s="8" t="inlineStr">
@@ -9140,7 +9140,7 @@
       </c>
       <c r="F69" s="8" t="inlineStr">
         <is>
-          <t>Sub-Head - IX, Plastering</t>
+          <t>Sub-Head - III, R.C.C. Work</t>
         </is>
       </c>
       <c r="G69" s="8" t="inlineStr">
@@ -9502,7 +9502,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Sub-Head - X, White/Colour Washing &amp; Painting</t>
+          <t>Sub-Head - V, Wood Work</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -9950,7 +9950,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Sub-Head - XI, Sundry Items / Site Development</t>
+          <t>Sub-Head - II, Cement Concrete Work</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">

</xml_diff>